<commit_message>
descarga excel y pdf actas
</commit_message>
<xml_diff>
--- a/app/Documents/formatoActaConformidad.xlsx
+++ b/app/Documents/formatoActaConformidad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GIAN AVALO\Downloads\git (3)\app\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BC9220-BAF4-4D96-8D28-B0EBCD991852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA152B20-5F58-492D-8397-47FCFDF5A4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="832" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1710,6 +1710,18 @@
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2180,18 +2192,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2785,14 +2785,14 @@
       <c r="A2" s="22"/>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
-      <c r="D2" s="115" t="s">
+      <c r="D2" s="119" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="115"/>
-      <c r="F2" s="115"/>
-      <c r="G2" s="115"/>
-      <c r="H2" s="115"/>
-      <c r="I2" s="115"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="119"/>
+      <c r="H2" s="119"/>
+      <c r="I2" s="119"/>
       <c r="J2" s="24"/>
       <c r="K2" s="25"/>
       <c r="L2" s="26"/>
@@ -2800,15 +2800,15 @@
     <row r="3" spans="1:15" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="18"/>
       <c r="B3" s="19"/>
-      <c r="C3" s="123" t="s">
+      <c r="C3" s="127" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
-      <c r="I3" s="124"/>
+      <c r="D3" s="127"/>
+      <c r="E3" s="127"/>
+      <c r="F3" s="127"/>
+      <c r="G3" s="127"/>
+      <c r="H3" s="127"/>
+      <c r="I3" s="128"/>
       <c r="J3" s="45" t="s">
         <v>2</v>
       </c>
@@ -2820,13 +2820,13 @@
     <row r="4" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="20"/>
       <c r="B4" s="21"/>
-      <c r="C4" s="123"/>
-      <c r="D4" s="123"/>
-      <c r="E4" s="123"/>
-      <c r="F4" s="123"/>
-      <c r="G4" s="123"/>
-      <c r="H4" s="123"/>
-      <c r="I4" s="124"/>
+      <c r="C4" s="127"/>
+      <c r="D4" s="127"/>
+      <c r="E4" s="127"/>
+      <c r="F4" s="127"/>
+      <c r="G4" s="127"/>
+      <c r="H4" s="127"/>
+      <c r="I4" s="128"/>
       <c r="J4" s="45" t="s">
         <v>4</v>
       </c>
@@ -2836,73 +2836,73 @@
       <c r="L4" s="14"/>
     </row>
     <row r="5" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="126"/>
-      <c r="B5" s="127"/>
-      <c r="C5" s="127"/>
-      <c r="D5" s="127"/>
-      <c r="E5" s="127"/>
-      <c r="F5" s="127"/>
-      <c r="G5" s="127"/>
-      <c r="H5" s="127"/>
-      <c r="I5" s="127"/>
-      <c r="J5" s="127"/>
-      <c r="K5" s="128"/>
+      <c r="A5" s="130"/>
+      <c r="B5" s="131"/>
+      <c r="C5" s="131"/>
+      <c r="D5" s="131"/>
+      <c r="E5" s="131"/>
+      <c r="F5" s="131"/>
+      <c r="G5" s="131"/>
+      <c r="H5" s="131"/>
+      <c r="I5" s="131"/>
+      <c r="J5" s="131"/>
+      <c r="K5" s="132"/>
       <c r="L5" s="14"/>
     </row>
     <row r="6" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="113" t="s">
+      <c r="A6" s="117" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="114"/>
-      <c r="C6" s="114"/>
-      <c r="D6" s="114"/>
-      <c r="E6" s="114"/>
-      <c r="F6" s="120" t="s">
+      <c r="B6" s="118"/>
+      <c r="C6" s="118"/>
+      <c r="D6" s="118"/>
+      <c r="E6" s="118"/>
+      <c r="F6" s="124" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="120"/>
-      <c r="H6" s="121" t="s">
+      <c r="G6" s="124"/>
+      <c r="H6" s="125" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="122"/>
-      <c r="J6" s="122"/>
-      <c r="K6" s="122"/>
+      <c r="I6" s="126"/>
+      <c r="J6" s="126"/>
+      <c r="K6" s="126"/>
       <c r="L6" s="14"/>
     </row>
     <row r="7" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="116"/>
-      <c r="B7" s="117"/>
-      <c r="C7" s="117"/>
-      <c r="D7" s="117"/>
-      <c r="E7" s="117"/>
-      <c r="F7" s="125" t="s">
+      <c r="A7" s="120"/>
+      <c r="B7" s="121"/>
+      <c r="C7" s="121"/>
+      <c r="D7" s="121"/>
+      <c r="E7" s="121"/>
+      <c r="F7" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="125"/>
-      <c r="H7" s="121" t="s">
+      <c r="G7" s="129"/>
+      <c r="H7" s="125" t="s">
         <v>9</v>
       </c>
-      <c r="I7" s="122"/>
-      <c r="J7" s="122"/>
-      <c r="K7" s="122"/>
+      <c r="I7" s="126"/>
+      <c r="J7" s="126"/>
+      <c r="K7" s="126"/>
       <c r="L7" s="14"/>
     </row>
     <row r="8" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="118"/>
-      <c r="B8" s="119"/>
-      <c r="C8" s="119"/>
-      <c r="D8" s="119"/>
-      <c r="E8" s="119"/>
-      <c r="F8" s="125" t="s">
+      <c r="A8" s="122"/>
+      <c r="B8" s="123"/>
+      <c r="C8" s="123"/>
+      <c r="D8" s="123"/>
+      <c r="E8" s="123"/>
+      <c r="F8" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="125"/>
-      <c r="H8" s="121" t="s">
+      <c r="G8" s="129"/>
+      <c r="H8" s="125" t="s">
         <v>9</v>
       </c>
-      <c r="I8" s="122"/>
-      <c r="J8" s="122"/>
-      <c r="K8" s="122"/>
+      <c r="I8" s="126"/>
+      <c r="J8" s="126"/>
+      <c r="K8" s="126"/>
       <c r="L8" s="14"/>
     </row>
     <row r="9" spans="1:15" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2920,21 +2920,21 @@
       <c r="L9" s="14"/>
     </row>
     <row r="10" spans="1:15" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="113" t="s">
+      <c r="A10" s="117" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="114"/>
-      <c r="C10" s="114"/>
-      <c r="D10" s="114"/>
-      <c r="E10" s="114"/>
-      <c r="F10" s="121" t="s">
+      <c r="B10" s="118"/>
+      <c r="C10" s="118"/>
+      <c r="D10" s="118"/>
+      <c r="E10" s="118"/>
+      <c r="F10" s="125" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="122"/>
-      <c r="H10" s="122"/>
-      <c r="I10" s="122"/>
-      <c r="J10" s="122"/>
-      <c r="K10" s="129"/>
+      <c r="G10" s="126"/>
+      <c r="H10" s="126"/>
+      <c r="I10" s="126"/>
+      <c r="J10" s="126"/>
+      <c r="K10" s="133"/>
       <c r="L10" s="14"/>
     </row>
     <row r="11" spans="1:15" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2952,44 +2952,44 @@
       <c r="L11" s="14"/>
     </row>
     <row r="12" spans="1:15" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="163" t="s">
+      <c r="A12" s="167" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="164"/>
-      <c r="C12" s="164"/>
-      <c r="D12" s="164"/>
-      <c r="E12" s="165"/>
-      <c r="F12" s="172" t="s">
+      <c r="B12" s="168"/>
+      <c r="C12" s="168"/>
+      <c r="D12" s="168"/>
+      <c r="E12" s="169"/>
+      <c r="F12" s="176" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="122"/>
-      <c r="H12" s="122"/>
-      <c r="I12" s="122"/>
-      <c r="J12" s="122"/>
-      <c r="K12" s="129"/>
-      <c r="L12" s="159"/>
-      <c r="M12" s="160"/>
-      <c r="N12" s="160"/>
-      <c r="O12" s="160"/>
+      <c r="G12" s="126"/>
+      <c r="H12" s="126"/>
+      <c r="I12" s="126"/>
+      <c r="J12" s="126"/>
+      <c r="K12" s="133"/>
+      <c r="L12" s="163"/>
+      <c r="M12" s="164"/>
+      <c r="N12" s="164"/>
+      <c r="O12" s="164"/>
     </row>
     <row r="13" spans="1:15" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="169"/>
-      <c r="B13" s="170"/>
-      <c r="C13" s="170"/>
-      <c r="D13" s="170"/>
-      <c r="E13" s="171"/>
-      <c r="F13" s="172" t="s">
+      <c r="A13" s="173"/>
+      <c r="B13" s="174"/>
+      <c r="C13" s="174"/>
+      <c r="D13" s="174"/>
+      <c r="E13" s="175"/>
+      <c r="F13" s="176" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="122"/>
-      <c r="H13" s="122"/>
-      <c r="I13" s="122"/>
-      <c r="J13" s="122"/>
-      <c r="K13" s="129"/>
-      <c r="L13" s="159"/>
-      <c r="M13" s="160"/>
-      <c r="N13" s="160"/>
-      <c r="O13" s="160"/>
+      <c r="G13" s="126"/>
+      <c r="H13" s="126"/>
+      <c r="I13" s="126"/>
+      <c r="J13" s="126"/>
+      <c r="K13" s="133"/>
+      <c r="L13" s="163"/>
+      <c r="M13" s="164"/>
+      <c r="N13" s="164"/>
+      <c r="O13" s="164"/>
     </row>
     <row r="14" spans="1:15" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="15"/>
@@ -3006,19 +3006,19 @@
       <c r="L14" s="14"/>
     </row>
     <row r="15" spans="1:15" s="2" customFormat="1" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="163" t="s">
+      <c r="A15" s="167" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="164"/>
-      <c r="C15" s="164"/>
-      <c r="D15" s="164"/>
-      <c r="E15" s="165"/>
-      <c r="F15" s="173" t="s">
+      <c r="B15" s="168"/>
+      <c r="C15" s="168"/>
+      <c r="D15" s="168"/>
+      <c r="E15" s="169"/>
+      <c r="F15" s="177" t="s">
         <v>17</v>
       </c>
-      <c r="G15" s="174"/>
-      <c r="H15" s="174"/>
-      <c r="I15" s="175"/>
+      <c r="G15" s="178"/>
+      <c r="H15" s="178"/>
+      <c r="I15" s="179"/>
       <c r="J15" s="47" t="s">
         <v>18</v>
       </c>
@@ -3028,17 +3028,17 @@
       <c r="L15" s="14"/>
     </row>
     <row r="16" spans="1:15" s="2" customFormat="1" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="166"/>
-      <c r="B16" s="167"/>
-      <c r="C16" s="167"/>
-      <c r="D16" s="167"/>
-      <c r="E16" s="168"/>
-      <c r="F16" s="173" t="s">
+      <c r="A16" s="170"/>
+      <c r="B16" s="171"/>
+      <c r="C16" s="171"/>
+      <c r="D16" s="171"/>
+      <c r="E16" s="172"/>
+      <c r="F16" s="177" t="s">
         <v>20</v>
       </c>
-      <c r="G16" s="174"/>
-      <c r="H16" s="174"/>
-      <c r="I16" s="175"/>
+      <c r="G16" s="178"/>
+      <c r="H16" s="178"/>
+      <c r="I16" s="179"/>
       <c r="J16" s="47" t="s">
         <v>18</v>
       </c>
@@ -3048,17 +3048,17 @@
       <c r="L16" s="14"/>
     </row>
     <row r="17" spans="1:12" s="2" customFormat="1" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="166"/>
-      <c r="B17" s="167"/>
-      <c r="C17" s="167"/>
-      <c r="D17" s="167"/>
-      <c r="E17" s="168"/>
-      <c r="F17" s="173" t="s">
+      <c r="A17" s="170"/>
+      <c r="B17" s="171"/>
+      <c r="C17" s="171"/>
+      <c r="D17" s="171"/>
+      <c r="E17" s="172"/>
+      <c r="F17" s="177" t="s">
         <v>21</v>
       </c>
-      <c r="G17" s="174"/>
-      <c r="H17" s="174"/>
-      <c r="I17" s="175"/>
+      <c r="G17" s="178"/>
+      <c r="H17" s="178"/>
+      <c r="I17" s="179"/>
       <c r="J17" s="47" t="s">
         <v>18</v>
       </c>
@@ -3068,19 +3068,19 @@
       <c r="L17" s="14"/>
     </row>
     <row r="18" spans="1:12" s="2" customFormat="1" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="169"/>
-      <c r="B18" s="170"/>
-      <c r="C18" s="170"/>
-      <c r="D18" s="170"/>
-      <c r="E18" s="171"/>
-      <c r="F18" s="176" t="s">
+      <c r="A18" s="173"/>
+      <c r="B18" s="174"/>
+      <c r="C18" s="174"/>
+      <c r="D18" s="174"/>
+      <c r="E18" s="175"/>
+      <c r="F18" s="180" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="177"/>
-      <c r="H18" s="177"/>
-      <c r="I18" s="177"/>
-      <c r="J18" s="177"/>
-      <c r="K18" s="178"/>
+      <c r="G18" s="181"/>
+      <c r="H18" s="181"/>
+      <c r="I18" s="181"/>
+      <c r="J18" s="181"/>
+      <c r="K18" s="182"/>
       <c r="L18" s="14"/>
     </row>
     <row r="19" spans="1:12" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3098,37 +3098,37 @@
       <c r="L19" s="14"/>
     </row>
     <row r="20" spans="1:12" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="136" t="s">
+      <c r="A20" s="140" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="137"/>
-      <c r="C20" s="130" t="s">
+      <c r="B20" s="141"/>
+      <c r="C20" s="134" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="131"/>
-      <c r="E20" s="131"/>
-      <c r="F20" s="131"/>
-      <c r="G20" s="131"/>
-      <c r="H20" s="131"/>
-      <c r="I20" s="131"/>
-      <c r="J20" s="131"/>
-      <c r="K20" s="132"/>
+      <c r="D20" s="135"/>
+      <c r="E20" s="135"/>
+      <c r="F20" s="135"/>
+      <c r="G20" s="135"/>
+      <c r="H20" s="135"/>
+      <c r="I20" s="135"/>
+      <c r="J20" s="135"/>
+      <c r="K20" s="136"/>
       <c r="L20" s="14"/>
     </row>
     <row r="21" spans="1:12" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="138"/>
-      <c r="B21" s="139"/>
-      <c r="C21" s="140" t="s">
+      <c r="A21" s="142"/>
+      <c r="B21" s="143"/>
+      <c r="C21" s="144" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="141"/>
-      <c r="E21" s="141"/>
-      <c r="F21" s="141"/>
-      <c r="G21" s="141"/>
-      <c r="H21" s="141"/>
-      <c r="I21" s="141"/>
-      <c r="J21" s="141"/>
-      <c r="K21" s="142"/>
+      <c r="D21" s="145"/>
+      <c r="E21" s="145"/>
+      <c r="F21" s="145"/>
+      <c r="G21" s="145"/>
+      <c r="H21" s="145"/>
+      <c r="I21" s="145"/>
+      <c r="J21" s="145"/>
+      <c r="K21" s="146"/>
       <c r="L21" s="14"/>
     </row>
     <row r="22" spans="1:12" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3146,65 +3146,65 @@
       <c r="L22" s="14"/>
     </row>
     <row r="23" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="136" t="s">
+      <c r="A23" s="140" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="143"/>
-      <c r="C23" s="145" t="s">
+      <c r="B23" s="147"/>
+      <c r="C23" s="149" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="146"/>
-      <c r="E23" s="146"/>
-      <c r="F23" s="146"/>
-      <c r="G23" s="146"/>
-      <c r="H23" s="146"/>
-      <c r="I23" s="146"/>
-      <c r="J23" s="146"/>
-      <c r="K23" s="147"/>
+      <c r="D23" s="150"/>
+      <c r="E23" s="150"/>
+      <c r="F23" s="150"/>
+      <c r="G23" s="150"/>
+      <c r="H23" s="150"/>
+      <c r="I23" s="150"/>
+      <c r="J23" s="150"/>
+      <c r="K23" s="151"/>
       <c r="L23" s="14"/>
     </row>
     <row r="24" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="138"/>
-      <c r="B24" s="144"/>
-      <c r="C24" s="148"/>
-      <c r="D24" s="149"/>
-      <c r="E24" s="149"/>
-      <c r="F24" s="149"/>
-      <c r="G24" s="149"/>
-      <c r="H24" s="149"/>
-      <c r="I24" s="149"/>
-      <c r="J24" s="149"/>
-      <c r="K24" s="150"/>
+      <c r="A24" s="142"/>
+      <c r="B24" s="148"/>
+      <c r="C24" s="152"/>
+      <c r="D24" s="153"/>
+      <c r="E24" s="153"/>
+      <c r="F24" s="153"/>
+      <c r="G24" s="153"/>
+      <c r="H24" s="153"/>
+      <c r="I24" s="153"/>
+      <c r="J24" s="153"/>
+      <c r="K24" s="154"/>
       <c r="L24" s="14"/>
     </row>
     <row r="25" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="151" t="s">
+      <c r="A25" s="155" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="152"/>
-      <c r="C25" s="152"/>
-      <c r="D25" s="152"/>
-      <c r="E25" s="152"/>
-      <c r="F25" s="152"/>
-      <c r="G25" s="152"/>
-      <c r="H25" s="152"/>
-      <c r="I25" s="152"/>
-      <c r="J25" s="152"/>
-      <c r="K25" s="153"/>
+      <c r="B25" s="156"/>
+      <c r="C25" s="156"/>
+      <c r="D25" s="156"/>
+      <c r="E25" s="156"/>
+      <c r="F25" s="156"/>
+      <c r="G25" s="156"/>
+      <c r="H25" s="156"/>
+      <c r="I25" s="156"/>
+      <c r="J25" s="156"/>
+      <c r="K25" s="157"/>
       <c r="L25" s="14"/>
     </row>
     <row r="26" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="154"/>
-      <c r="B26" s="155"/>
-      <c r="C26" s="155"/>
-      <c r="D26" s="155"/>
-      <c r="E26" s="155"/>
-      <c r="F26" s="155"/>
-      <c r="G26" s="155"/>
-      <c r="H26" s="155"/>
-      <c r="I26" s="155"/>
-      <c r="J26" s="155"/>
-      <c r="K26" s="156"/>
+      <c r="A26" s="158"/>
+      <c r="B26" s="159"/>
+      <c r="C26" s="159"/>
+      <c r="D26" s="159"/>
+      <c r="E26" s="159"/>
+      <c r="F26" s="159"/>
+      <c r="G26" s="159"/>
+      <c r="H26" s="159"/>
+      <c r="I26" s="159"/>
+      <c r="J26" s="159"/>
+      <c r="K26" s="160"/>
       <c r="L26" s="14"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
@@ -3223,12 +3223,12 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="32"/>
-      <c r="B28" s="161"/>
-      <c r="C28" s="161"/>
-      <c r="D28" s="161"/>
-      <c r="E28" s="161"/>
-      <c r="F28" s="161"/>
-      <c r="G28" s="161"/>
+      <c r="B28" s="165"/>
+      <c r="C28" s="165"/>
+      <c r="D28" s="165"/>
+      <c r="E28" s="165"/>
+      <c r="F28" s="165"/>
+      <c r="G28" s="165"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
       <c r="J28" s="33"/>
@@ -3294,36 +3294,36 @@
     <row r="33" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="35"/>
       <c r="B33" s="36"/>
-      <c r="C33" s="157" t="s">
+      <c r="C33" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="D33" s="157"/>
-      <c r="E33" s="157"/>
-      <c r="F33" s="157"/>
+      <c r="D33" s="161"/>
+      <c r="E33" s="161"/>
+      <c r="F33" s="161"/>
       <c r="G33" s="38"/>
-      <c r="H33" s="157" t="s">
+      <c r="H33" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="I33" s="157"/>
-      <c r="J33" s="157"/>
+      <c r="I33" s="161"/>
+      <c r="J33" s="161"/>
       <c r="K33" s="39"/>
       <c r="L33" s="14"/>
     </row>
     <row r="34" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="35"/>
       <c r="B34" s="36"/>
-      <c r="C34" s="158" t="s">
+      <c r="C34" s="162" t="s">
         <v>30</v>
       </c>
-      <c r="D34" s="158"/>
-      <c r="E34" s="158"/>
-      <c r="F34" s="158"/>
+      <c r="D34" s="162"/>
+      <c r="E34" s="162"/>
+      <c r="F34" s="162"/>
       <c r="G34" s="38"/>
-      <c r="H34" s="158" t="s">
+      <c r="H34" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="I34" s="158"/>
-      <c r="J34" s="158"/>
+      <c r="I34" s="162"/>
+      <c r="J34" s="162"/>
       <c r="K34" s="39"/>
       <c r="L34" s="14"/>
     </row>
@@ -3335,11 +3335,11 @@
       <c r="E35" s="38"/>
       <c r="F35" s="38"/>
       <c r="G35" s="38"/>
-      <c r="H35" s="162" t="s">
+      <c r="H35" s="166" t="s">
         <v>32</v>
       </c>
-      <c r="I35" s="162"/>
-      <c r="J35" s="162"/>
+      <c r="I35" s="166"/>
+      <c r="J35" s="166"/>
       <c r="K35" s="39"/>
       <c r="L35" s="14"/>
     </row>
@@ -3358,35 +3358,35 @@
       <c r="L36" s="14"/>
     </row>
     <row r="37" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="130" t="s">
+      <c r="A37" s="134" t="s">
         <v>33</v>
       </c>
-      <c r="B37" s="131"/>
-      <c r="C37" s="131"/>
-      <c r="D37" s="131"/>
-      <c r="E37" s="131"/>
-      <c r="F37" s="131"/>
-      <c r="G37" s="131"/>
-      <c r="H37" s="131"/>
-      <c r="I37" s="131"/>
-      <c r="J37" s="131"/>
-      <c r="K37" s="132"/>
+      <c r="B37" s="135"/>
+      <c r="C37" s="135"/>
+      <c r="D37" s="135"/>
+      <c r="E37" s="135"/>
+      <c r="F37" s="135"/>
+      <c r="G37" s="135"/>
+      <c r="H37" s="135"/>
+      <c r="I37" s="135"/>
+      <c r="J37" s="135"/>
+      <c r="K37" s="136"/>
       <c r="L37" s="14"/>
     </row>
     <row r="38" spans="1:12" ht="86.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="133" t="s">
+      <c r="A38" s="137" t="s">
         <v>34</v>
       </c>
-      <c r="B38" s="134"/>
-      <c r="C38" s="134"/>
-      <c r="D38" s="134"/>
-      <c r="E38" s="134"/>
-      <c r="F38" s="134"/>
-      <c r="G38" s="134"/>
-      <c r="H38" s="134"/>
-      <c r="I38" s="134"/>
-      <c r="J38" s="134"/>
-      <c r="K38" s="135"/>
+      <c r="B38" s="138"/>
+      <c r="C38" s="138"/>
+      <c r="D38" s="138"/>
+      <c r="E38" s="138"/>
+      <c r="F38" s="138"/>
+      <c r="G38" s="138"/>
+      <c r="H38" s="138"/>
+      <c r="I38" s="138"/>
+      <c r="J38" s="138"/>
+      <c r="K38" s="139"/>
       <c r="L38" s="14"/>
     </row>
   </sheetData>
@@ -3466,14 +3466,14 @@
       <c r="A2" s="69"/>
       <c r="B2" s="69"/>
       <c r="C2" s="69"/>
-      <c r="D2" s="182" t="s">
+      <c r="D2" s="186" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="182"/>
-      <c r="F2" s="182"/>
-      <c r="G2" s="182"/>
-      <c r="H2" s="182"/>
-      <c r="I2" s="182"/>
+      <c r="E2" s="186"/>
+      <c r="F2" s="186"/>
+      <c r="G2" s="186"/>
+      <c r="H2" s="186"/>
+      <c r="I2" s="186"/>
       <c r="J2" s="70"/>
       <c r="K2" s="71"/>
       <c r="L2" s="26"/>
@@ -3482,29 +3482,29 @@
       <c r="A3" s="19"/>
       <c r="B3" s="19"/>
       <c r="C3" s="72"/>
-      <c r="D3" s="189" t="s">
+      <c r="D3" s="193" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="189"/>
-      <c r="F3" s="189"/>
-      <c r="G3" s="189"/>
-      <c r="H3" s="189"/>
-      <c r="I3" s="189"/>
+      <c r="E3" s="193"/>
+      <c r="F3" s="193"/>
+      <c r="G3" s="193"/>
+      <c r="H3" s="193"/>
+      <c r="I3" s="193"/>
       <c r="J3" s="14"/>
       <c r="L3"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="127"/>
-      <c r="B4" s="127"/>
-      <c r="C4" s="127"/>
-      <c r="D4" s="127"/>
-      <c r="E4" s="127"/>
-      <c r="F4" s="127"/>
-      <c r="G4" s="127"/>
-      <c r="H4" s="127"/>
-      <c r="I4" s="127"/>
-      <c r="J4" s="127"/>
-      <c r="K4" s="127"/>
+      <c r="A4" s="131"/>
+      <c r="B4" s="131"/>
+      <c r="C4" s="131"/>
+      <c r="D4" s="131"/>
+      <c r="E4" s="131"/>
+      <c r="F4" s="131"/>
+      <c r="G4" s="131"/>
+      <c r="H4" s="131"/>
+      <c r="I4" s="131"/>
+      <c r="J4" s="131"/>
+      <c r="K4" s="131"/>
       <c r="L4" s="14"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -3690,53 +3690,53 @@
       <c r="L17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="183" t="s">
+      <c r="A18" s="187" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="184"/>
-      <c r="C18" s="184"/>
-      <c r="D18" s="184"/>
-      <c r="E18" s="184"/>
-      <c r="F18" s="185" t="s">
+      <c r="B18" s="188"/>
+      <c r="C18" s="188"/>
+      <c r="D18" s="188"/>
+      <c r="E18" s="188"/>
+      <c r="F18" s="189" t="s">
         <v>6</v>
       </c>
-      <c r="G18" s="185"/>
-      <c r="H18" s="186"/>
-      <c r="I18" s="187"/>
-      <c r="J18" s="187"/>
-      <c r="K18" s="188"/>
+      <c r="G18" s="189"/>
+      <c r="H18" s="190"/>
+      <c r="I18" s="191"/>
+      <c r="J18" s="191"/>
+      <c r="K18" s="192"/>
       <c r="L18" s="14"/>
     </row>
     <row r="19" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="116"/>
-      <c r="B19" s="117"/>
-      <c r="C19" s="117"/>
-      <c r="D19" s="117"/>
-      <c r="E19" s="117"/>
-      <c r="F19" s="125" t="s">
+      <c r="A19" s="120"/>
+      <c r="B19" s="121"/>
+      <c r="C19" s="121"/>
+      <c r="D19" s="121"/>
+      <c r="E19" s="121"/>
+      <c r="F19" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="G19" s="125"/>
-      <c r="H19" s="121"/>
-      <c r="I19" s="122"/>
-      <c r="J19" s="122"/>
-      <c r="K19" s="129"/>
+      <c r="G19" s="129"/>
+      <c r="H19" s="125"/>
+      <c r="I19" s="126"/>
+      <c r="J19" s="126"/>
+      <c r="K19" s="133"/>
       <c r="L19" s="14"/>
     </row>
     <row r="20" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="118"/>
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="125" t="s">
+      <c r="A20" s="122"/>
+      <c r="B20" s="123"/>
+      <c r="C20" s="123"/>
+      <c r="D20" s="123"/>
+      <c r="E20" s="123"/>
+      <c r="F20" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="G20" s="125"/>
-      <c r="H20" s="121"/>
-      <c r="I20" s="122"/>
-      <c r="J20" s="122"/>
-      <c r="K20" s="129"/>
+      <c r="G20" s="129"/>
+      <c r="H20" s="125"/>
+      <c r="I20" s="126"/>
+      <c r="J20" s="126"/>
+      <c r="K20" s="133"/>
       <c r="L20" s="14"/>
     </row>
     <row r="21" spans="1:15" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3754,19 +3754,19 @@
       <c r="L21" s="14"/>
     </row>
     <row r="22" spans="1:15" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="113" t="s">
+      <c r="A22" s="117" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="114"/>
-      <c r="C22" s="114"/>
-      <c r="D22" s="114"/>
-      <c r="E22" s="114"/>
-      <c r="F22" s="121"/>
-      <c r="G22" s="122"/>
-      <c r="H22" s="122"/>
-      <c r="I22" s="122"/>
-      <c r="J22" s="122"/>
-      <c r="K22" s="129"/>
+      <c r="B22" s="118"/>
+      <c r="C22" s="118"/>
+      <c r="D22" s="118"/>
+      <c r="E22" s="118"/>
+      <c r="F22" s="125"/>
+      <c r="G22" s="126"/>
+      <c r="H22" s="126"/>
+      <c r="I22" s="126"/>
+      <c r="J22" s="126"/>
+      <c r="K22" s="133"/>
       <c r="L22" s="14"/>
     </row>
     <row r="23" spans="1:15" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3784,40 +3784,40 @@
       <c r="L23" s="14"/>
     </row>
     <row r="24" spans="1:15" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="163" t="s">
+      <c r="A24" s="167" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="164"/>
-      <c r="C24" s="164"/>
-      <c r="D24" s="164"/>
-      <c r="E24" s="165"/>
-      <c r="F24" s="172"/>
-      <c r="G24" s="122"/>
-      <c r="H24" s="122"/>
-      <c r="I24" s="122"/>
-      <c r="J24" s="122"/>
-      <c r="K24" s="129"/>
-      <c r="L24" s="159"/>
-      <c r="M24" s="160"/>
-      <c r="N24" s="160"/>
-      <c r="O24" s="160"/>
+      <c r="B24" s="168"/>
+      <c r="C24" s="168"/>
+      <c r="D24" s="168"/>
+      <c r="E24" s="169"/>
+      <c r="F24" s="176"/>
+      <c r="G24" s="126"/>
+      <c r="H24" s="126"/>
+      <c r="I24" s="126"/>
+      <c r="J24" s="126"/>
+      <c r="K24" s="133"/>
+      <c r="L24" s="163"/>
+      <c r="M24" s="164"/>
+      <c r="N24" s="164"/>
+      <c r="O24" s="164"/>
     </row>
     <row r="25" spans="1:15" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="169"/>
-      <c r="B25" s="170"/>
-      <c r="C25" s="170"/>
-      <c r="D25" s="170"/>
-      <c r="E25" s="171"/>
-      <c r="F25" s="172"/>
-      <c r="G25" s="122"/>
-      <c r="H25" s="122"/>
-      <c r="I25" s="122"/>
-      <c r="J25" s="122"/>
-      <c r="K25" s="129"/>
-      <c r="L25" s="159"/>
-      <c r="M25" s="160"/>
-      <c r="N25" s="160"/>
-      <c r="O25" s="160"/>
+      <c r="A25" s="173"/>
+      <c r="B25" s="174"/>
+      <c r="C25" s="174"/>
+      <c r="D25" s="174"/>
+      <c r="E25" s="175"/>
+      <c r="F25" s="176"/>
+      <c r="G25" s="126"/>
+      <c r="H25" s="126"/>
+      <c r="I25" s="126"/>
+      <c r="J25" s="126"/>
+      <c r="K25" s="133"/>
+      <c r="L25" s="163"/>
+      <c r="M25" s="164"/>
+      <c r="N25" s="164"/>
+      <c r="O25" s="164"/>
     </row>
     <row r="26" spans="1:15" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="15"/>
@@ -3834,19 +3834,19 @@
       <c r="L26" s="14"/>
     </row>
     <row r="27" spans="1:15" s="2" customFormat="1" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="163" t="s">
+      <c r="A27" s="167" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="164"/>
-      <c r="C27" s="164"/>
-      <c r="D27" s="164"/>
-      <c r="E27" s="165"/>
-      <c r="F27" s="173" t="s">
+      <c r="B27" s="168"/>
+      <c r="C27" s="168"/>
+      <c r="D27" s="168"/>
+      <c r="E27" s="169"/>
+      <c r="F27" s="177" t="s">
         <v>17</v>
       </c>
-      <c r="G27" s="174"/>
-      <c r="H27" s="174"/>
-      <c r="I27" s="175"/>
+      <c r="G27" s="178"/>
+      <c r="H27" s="178"/>
+      <c r="I27" s="179"/>
       <c r="J27" s="47" t="s">
         <v>18</v>
       </c>
@@ -3856,17 +3856,17 @@
       <c r="L27" s="14"/>
     </row>
     <row r="28" spans="1:15" s="2" customFormat="1" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="166"/>
-      <c r="B28" s="167"/>
-      <c r="C28" s="167"/>
-      <c r="D28" s="167"/>
-      <c r="E28" s="168"/>
-      <c r="F28" s="173" t="s">
+      <c r="A28" s="170"/>
+      <c r="B28" s="171"/>
+      <c r="C28" s="171"/>
+      <c r="D28" s="171"/>
+      <c r="E28" s="172"/>
+      <c r="F28" s="177" t="s">
         <v>20</v>
       </c>
-      <c r="G28" s="174"/>
-      <c r="H28" s="174"/>
-      <c r="I28" s="175"/>
+      <c r="G28" s="178"/>
+      <c r="H28" s="178"/>
+      <c r="I28" s="179"/>
       <c r="J28" s="47" t="s">
         <v>18</v>
       </c>
@@ -3876,17 +3876,17 @@
       <c r="L28" s="14"/>
     </row>
     <row r="29" spans="1:15" s="2" customFormat="1" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="166"/>
-      <c r="B29" s="167"/>
-      <c r="C29" s="167"/>
-      <c r="D29" s="167"/>
-      <c r="E29" s="168"/>
-      <c r="F29" s="173" t="s">
+      <c r="A29" s="170"/>
+      <c r="B29" s="171"/>
+      <c r="C29" s="171"/>
+      <c r="D29" s="171"/>
+      <c r="E29" s="172"/>
+      <c r="F29" s="177" t="s">
         <v>21</v>
       </c>
-      <c r="G29" s="174"/>
-      <c r="H29" s="174"/>
-      <c r="I29" s="175"/>
+      <c r="G29" s="178"/>
+      <c r="H29" s="178"/>
+      <c r="I29" s="179"/>
       <c r="J29" s="47" t="s">
         <v>18</v>
       </c>
@@ -3896,19 +3896,19 @@
       <c r="L29" s="14"/>
     </row>
     <row r="30" spans="1:15" s="2" customFormat="1" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="169"/>
-      <c r="B30" s="170"/>
-      <c r="C30" s="170"/>
-      <c r="D30" s="170"/>
-      <c r="E30" s="171"/>
-      <c r="F30" s="179" t="s">
+      <c r="A30" s="173"/>
+      <c r="B30" s="174"/>
+      <c r="C30" s="174"/>
+      <c r="D30" s="174"/>
+      <c r="E30" s="175"/>
+      <c r="F30" s="183" t="s">
         <v>22</v>
       </c>
-      <c r="G30" s="180"/>
-      <c r="H30" s="180"/>
-      <c r="I30" s="180"/>
-      <c r="J30" s="180"/>
-      <c r="K30" s="181"/>
+      <c r="G30" s="184"/>
+      <c r="H30" s="184"/>
+      <c r="I30" s="184"/>
+      <c r="J30" s="184"/>
+      <c r="K30" s="185"/>
       <c r="L30" s="14"/>
     </row>
     <row r="31" spans="1:15" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3926,35 +3926,35 @@
       <c r="L31" s="14"/>
     </row>
     <row r="32" spans="1:15" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="136" t="s">
+      <c r="A32" s="140" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="137"/>
-      <c r="C32" s="130" t="s">
+      <c r="B32" s="141"/>
+      <c r="C32" s="134" t="s">
         <v>24</v>
       </c>
-      <c r="D32" s="131"/>
-      <c r="E32" s="131"/>
-      <c r="F32" s="131"/>
-      <c r="G32" s="131"/>
-      <c r="H32" s="131"/>
-      <c r="I32" s="131"/>
-      <c r="J32" s="131"/>
-      <c r="K32" s="132"/>
+      <c r="D32" s="135"/>
+      <c r="E32" s="135"/>
+      <c r="F32" s="135"/>
+      <c r="G32" s="135"/>
+      <c r="H32" s="135"/>
+      <c r="I32" s="135"/>
+      <c r="J32" s="135"/>
+      <c r="K32" s="136"/>
       <c r="L32" s="14"/>
     </row>
     <row r="33" spans="1:12" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="138"/>
-      <c r="B33" s="139"/>
-      <c r="C33" s="140"/>
-      <c r="D33" s="141"/>
-      <c r="E33" s="141"/>
-      <c r="F33" s="141"/>
-      <c r="G33" s="141"/>
-      <c r="H33" s="141"/>
-      <c r="I33" s="141"/>
-      <c r="J33" s="141"/>
-      <c r="K33" s="142"/>
+      <c r="A33" s="142"/>
+      <c r="B33" s="143"/>
+      <c r="C33" s="144"/>
+      <c r="D33" s="145"/>
+      <c r="E33" s="145"/>
+      <c r="F33" s="145"/>
+      <c r="G33" s="145"/>
+      <c r="H33" s="145"/>
+      <c r="I33" s="145"/>
+      <c r="J33" s="145"/>
+      <c r="K33" s="146"/>
       <c r="L33" s="14"/>
     </row>
     <row r="34" spans="1:12" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3972,63 +3972,63 @@
       <c r="L34" s="14"/>
     </row>
     <row r="35" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="136" t="s">
+      <c r="A35" s="140" t="s">
         <v>26</v>
       </c>
-      <c r="B35" s="143"/>
-      <c r="C35" s="145" t="s">
+      <c r="B35" s="147"/>
+      <c r="C35" s="149" t="s">
         <v>27</v>
       </c>
-      <c r="D35" s="146"/>
-      <c r="E35" s="146"/>
-      <c r="F35" s="146"/>
-      <c r="G35" s="146"/>
-      <c r="H35" s="146"/>
-      <c r="I35" s="146"/>
-      <c r="J35" s="146"/>
-      <c r="K35" s="147"/>
+      <c r="D35" s="150"/>
+      <c r="E35" s="150"/>
+      <c r="F35" s="150"/>
+      <c r="G35" s="150"/>
+      <c r="H35" s="150"/>
+      <c r="I35" s="150"/>
+      <c r="J35" s="150"/>
+      <c r="K35" s="151"/>
       <c r="L35" s="14"/>
     </row>
     <row r="36" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="138"/>
-      <c r="B36" s="144"/>
-      <c r="C36" s="148"/>
-      <c r="D36" s="149"/>
-      <c r="E36" s="149"/>
-      <c r="F36" s="149"/>
-      <c r="G36" s="149"/>
-      <c r="H36" s="149"/>
-      <c r="I36" s="149"/>
-      <c r="J36" s="149"/>
-      <c r="K36" s="150"/>
+      <c r="A36" s="142"/>
+      <c r="B36" s="148"/>
+      <c r="C36" s="152"/>
+      <c r="D36" s="153"/>
+      <c r="E36" s="153"/>
+      <c r="F36" s="153"/>
+      <c r="G36" s="153"/>
+      <c r="H36" s="153"/>
+      <c r="I36" s="153"/>
+      <c r="J36" s="153"/>
+      <c r="K36" s="154"/>
       <c r="L36" s="14"/>
     </row>
     <row r="37" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="151"/>
-      <c r="B37" s="152"/>
-      <c r="C37" s="152"/>
-      <c r="D37" s="152"/>
-      <c r="E37" s="152"/>
-      <c r="F37" s="152"/>
-      <c r="G37" s="152"/>
-      <c r="H37" s="152"/>
-      <c r="I37" s="152"/>
-      <c r="J37" s="152"/>
-      <c r="K37" s="153"/>
+      <c r="A37" s="155"/>
+      <c r="B37" s="156"/>
+      <c r="C37" s="156"/>
+      <c r="D37" s="156"/>
+      <c r="E37" s="156"/>
+      <c r="F37" s="156"/>
+      <c r="G37" s="156"/>
+      <c r="H37" s="156"/>
+      <c r="I37" s="156"/>
+      <c r="J37" s="156"/>
+      <c r="K37" s="157"/>
       <c r="L37" s="14"/>
     </row>
     <row r="38" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="154"/>
-      <c r="B38" s="155"/>
-      <c r="C38" s="155"/>
-      <c r="D38" s="155"/>
-      <c r="E38" s="155"/>
-      <c r="F38" s="155"/>
-      <c r="G38" s="155"/>
-      <c r="H38" s="155"/>
-      <c r="I38" s="155"/>
-      <c r="J38" s="155"/>
-      <c r="K38" s="156"/>
+      <c r="A38" s="158"/>
+      <c r="B38" s="159"/>
+      <c r="C38" s="159"/>
+      <c r="D38" s="159"/>
+      <c r="E38" s="159"/>
+      <c r="F38" s="159"/>
+      <c r="G38" s="159"/>
+      <c r="H38" s="159"/>
+      <c r="I38" s="159"/>
+      <c r="J38" s="159"/>
+      <c r="K38" s="160"/>
       <c r="L38" s="14"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
@@ -4047,12 +4047,12 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="32"/>
-      <c r="B40" s="161"/>
-      <c r="C40" s="161"/>
-      <c r="D40" s="161"/>
-      <c r="E40" s="161"/>
-      <c r="F40" s="161"/>
-      <c r="G40" s="161"/>
+      <c r="B40" s="165"/>
+      <c r="C40" s="165"/>
+      <c r="D40" s="165"/>
+      <c r="E40" s="165"/>
+      <c r="F40" s="165"/>
+      <c r="G40" s="165"/>
       <c r="H40" s="33"/>
       <c r="I40" s="33"/>
       <c r="J40" s="33"/>
@@ -4118,36 +4118,36 @@
     <row r="45" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="35"/>
       <c r="B45" s="36"/>
-      <c r="C45" s="157" t="s">
+      <c r="C45" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="D45" s="157"/>
-      <c r="E45" s="157"/>
-      <c r="F45" s="157"/>
+      <c r="D45" s="161"/>
+      <c r="E45" s="161"/>
+      <c r="F45" s="161"/>
       <c r="G45" s="38"/>
-      <c r="H45" s="157" t="s">
+      <c r="H45" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="I45" s="157"/>
-      <c r="J45" s="157"/>
+      <c r="I45" s="161"/>
+      <c r="J45" s="161"/>
       <c r="K45" s="39"/>
       <c r="L45" s="14"/>
     </row>
     <row r="46" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="35"/>
       <c r="B46" s="36"/>
-      <c r="C46" s="158" t="s">
+      <c r="C46" s="162" t="s">
         <v>30</v>
       </c>
-      <c r="D46" s="158"/>
-      <c r="E46" s="158"/>
-      <c r="F46" s="158"/>
+      <c r="D46" s="162"/>
+      <c r="E46" s="162"/>
+      <c r="F46" s="162"/>
       <c r="G46" s="38"/>
-      <c r="H46" s="158" t="s">
+      <c r="H46" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="I46" s="158"/>
-      <c r="J46" s="158"/>
+      <c r="I46" s="162"/>
+      <c r="J46" s="162"/>
       <c r="K46" s="39"/>
       <c r="L46" s="14"/>
     </row>
@@ -4159,11 +4159,11 @@
       <c r="E47" s="38"/>
       <c r="F47" s="38"/>
       <c r="G47" s="38"/>
-      <c r="H47" s="162" t="s">
+      <c r="H47" s="166" t="s">
         <v>32</v>
       </c>
-      <c r="I47" s="162"/>
-      <c r="J47" s="162"/>
+      <c r="I47" s="166"/>
+      <c r="J47" s="166"/>
       <c r="K47" s="39"/>
       <c r="L47" s="14"/>
     </row>
@@ -4182,35 +4182,35 @@
       <c r="L48" s="14"/>
     </row>
     <row r="49" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="130" t="s">
+      <c r="A49" s="134" t="s">
         <v>33</v>
       </c>
-      <c r="B49" s="131"/>
-      <c r="C49" s="131"/>
-      <c r="D49" s="131"/>
-      <c r="E49" s="131"/>
-      <c r="F49" s="131"/>
-      <c r="G49" s="131"/>
-      <c r="H49" s="131"/>
-      <c r="I49" s="131"/>
-      <c r="J49" s="131"/>
-      <c r="K49" s="132"/>
+      <c r="B49" s="135"/>
+      <c r="C49" s="135"/>
+      <c r="D49" s="135"/>
+      <c r="E49" s="135"/>
+      <c r="F49" s="135"/>
+      <c r="G49" s="135"/>
+      <c r="H49" s="135"/>
+      <c r="I49" s="135"/>
+      <c r="J49" s="135"/>
+      <c r="K49" s="136"/>
       <c r="L49" s="14"/>
     </row>
     <row r="50" spans="1:12" ht="86.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="133" t="s">
+      <c r="A50" s="137" t="s">
         <v>34</v>
       </c>
-      <c r="B50" s="134"/>
-      <c r="C50" s="134"/>
-      <c r="D50" s="134"/>
-      <c r="E50" s="134"/>
-      <c r="F50" s="134"/>
-      <c r="G50" s="134"/>
-      <c r="H50" s="134"/>
-      <c r="I50" s="134"/>
-      <c r="J50" s="134"/>
-      <c r="K50" s="135"/>
+      <c r="B50" s="138"/>
+      <c r="C50" s="138"/>
+      <c r="D50" s="138"/>
+      <c r="E50" s="138"/>
+      <c r="F50" s="138"/>
+      <c r="G50" s="138"/>
+      <c r="H50" s="138"/>
+      <c r="I50" s="138"/>
+      <c r="J50" s="138"/>
+      <c r="K50" s="139"/>
       <c r="L50" s="14"/>
     </row>
   </sheetData>
@@ -4289,14 +4289,14 @@
       <c r="A2" s="22"/>
       <c r="B2" s="69"/>
       <c r="C2" s="69"/>
-      <c r="D2" s="199" t="s">
+      <c r="D2" s="203" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="199"/>
-      <c r="F2" s="199"/>
-      <c r="G2" s="199"/>
-      <c r="H2" s="199"/>
-      <c r="I2" s="199"/>
+      <c r="E2" s="203"/>
+      <c r="F2" s="203"/>
+      <c r="G2" s="203"/>
+      <c r="H2" s="203"/>
+      <c r="I2" s="203"/>
       <c r="J2" s="70"/>
       <c r="K2" s="71"/>
       <c r="L2" s="26"/>
@@ -4304,15 +4304,15 @@
     <row r="3" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18"/>
       <c r="B3" s="19"/>
-      <c r="C3" s="123" t="s">
+      <c r="C3" s="127" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
-      <c r="I3" s="123"/>
+      <c r="D3" s="127"/>
+      <c r="E3" s="127"/>
+      <c r="F3" s="127"/>
+      <c r="G3" s="127"/>
+      <c r="H3" s="127"/>
+      <c r="I3" s="127"/>
       <c r="J3" s="96" t="s">
         <v>38</v>
       </c>
@@ -4324,13 +4324,13 @@
     <row r="4" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="20"/>
       <c r="B4" s="21"/>
-      <c r="C4" s="123"/>
-      <c r="D4" s="123"/>
-      <c r="E4" s="123"/>
-      <c r="F4" s="123"/>
-      <c r="G4" s="123"/>
-      <c r="H4" s="123"/>
-      <c r="I4" s="123"/>
+      <c r="C4" s="127"/>
+      <c r="D4" s="127"/>
+      <c r="E4" s="127"/>
+      <c r="F4" s="127"/>
+      <c r="G4" s="127"/>
+      <c r="H4" s="127"/>
+      <c r="I4" s="127"/>
       <c r="J4" s="49" t="s">
         <v>40</v>
       </c>
@@ -4338,33 +4338,33 @@
       <c r="L4" s="14"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="126"/>
-      <c r="B5" s="127"/>
-      <c r="C5" s="127"/>
-      <c r="D5" s="127"/>
-      <c r="E5" s="127"/>
-      <c r="F5" s="127"/>
-      <c r="G5" s="127"/>
-      <c r="H5" s="127"/>
-      <c r="I5" s="127"/>
-      <c r="J5" s="127"/>
-      <c r="K5" s="128"/>
+      <c r="A5" s="130"/>
+      <c r="B5" s="131"/>
+      <c r="C5" s="131"/>
+      <c r="D5" s="131"/>
+      <c r="E5" s="131"/>
+      <c r="F5" s="131"/>
+      <c r="G5" s="131"/>
+      <c r="H5" s="131"/>
+      <c r="I5" s="131"/>
+      <c r="J5" s="131"/>
+      <c r="K5" s="132"/>
       <c r="L5" s="14"/>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="200" t="s">
+      <c r="A6" s="204" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="201"/>
-      <c r="C6" s="201"/>
-      <c r="D6" s="201"/>
-      <c r="E6" s="201"/>
-      <c r="F6" s="201"/>
-      <c r="G6" s="201"/>
-      <c r="H6" s="201"/>
-      <c r="I6" s="201"/>
-      <c r="J6" s="201"/>
-      <c r="K6" s="202"/>
+      <c r="B6" s="205"/>
+      <c r="C6" s="205"/>
+      <c r="D6" s="205"/>
+      <c r="E6" s="205"/>
+      <c r="F6" s="205"/>
+      <c r="G6" s="205"/>
+      <c r="H6" s="205"/>
+      <c r="I6" s="205"/>
+      <c r="J6" s="205"/>
+      <c r="K6" s="206"/>
       <c r="L6" s="14"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -4490,51 +4490,51 @@
       <c r="L14" s="14"/>
     </row>
     <row r="15" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="200" t="s">
+      <c r="A15" s="204" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="201"/>
-      <c r="C15" s="201"/>
-      <c r="D15" s="201"/>
-      <c r="E15" s="201"/>
-      <c r="F15" s="201"/>
-      <c r="G15" s="201"/>
-      <c r="H15" s="201"/>
-      <c r="I15" s="201"/>
-      <c r="J15" s="201"/>
-      <c r="K15" s="202"/>
+      <c r="B15" s="205"/>
+      <c r="C15" s="205"/>
+      <c r="D15" s="205"/>
+      <c r="E15" s="205"/>
+      <c r="F15" s="205"/>
+      <c r="G15" s="205"/>
+      <c r="H15" s="205"/>
+      <c r="I15" s="205"/>
+      <c r="J15" s="205"/>
+      <c r="K15" s="206"/>
       <c r="L15" s="14"/>
     </row>
     <row r="16" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="62"/>
-      <c r="B16" s="190" t="s">
+      <c r="B16" s="194" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="190"/>
+      <c r="C16" s="194"/>
       <c r="D16" s="63"/>
       <c r="E16" s="63"/>
       <c r="F16" s="63"/>
       <c r="G16" s="63"/>
-      <c r="H16" s="190" t="s">
+      <c r="H16" s="194" t="s">
         <v>49</v>
       </c>
-      <c r="I16" s="190"/>
+      <c r="I16" s="194"/>
       <c r="J16" s="63"/>
       <c r="K16" s="67"/>
       <c r="L16" s="14"/>
     </row>
     <row r="17" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="191"/>
-      <c r="B17" s="192"/>
-      <c r="C17" s="192"/>
-      <c r="D17" s="192"/>
-      <c r="E17" s="192"/>
-      <c r="F17" s="192"/>
-      <c r="G17" s="192"/>
-      <c r="H17" s="192"/>
-      <c r="I17" s="192"/>
-      <c r="J17" s="192"/>
-      <c r="K17" s="193"/>
+      <c r="A17" s="195"/>
+      <c r="B17" s="196"/>
+      <c r="C17" s="196"/>
+      <c r="D17" s="196"/>
+      <c r="E17" s="196"/>
+      <c r="F17" s="196"/>
+      <c r="G17" s="196"/>
+      <c r="H17" s="196"/>
+      <c r="I17" s="196"/>
+      <c r="J17" s="196"/>
+      <c r="K17" s="197"/>
       <c r="L17" s="14"/>
     </row>
     <row r="18" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4594,17 +4594,17 @@
       <c r="L21" s="14"/>
     </row>
     <row r="22" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="191"/>
-      <c r="B22" s="192"/>
-      <c r="C22" s="192"/>
-      <c r="D22" s="192"/>
-      <c r="E22" s="192"/>
-      <c r="F22" s="192"/>
-      <c r="G22" s="192"/>
-      <c r="H22" s="192"/>
-      <c r="I22" s="192"/>
-      <c r="J22" s="192"/>
-      <c r="K22" s="193"/>
+      <c r="A22" s="195"/>
+      <c r="B22" s="196"/>
+      <c r="C22" s="196"/>
+      <c r="D22" s="196"/>
+      <c r="E22" s="196"/>
+      <c r="F22" s="196"/>
+      <c r="G22" s="196"/>
+      <c r="H22" s="196"/>
+      <c r="I22" s="196"/>
+      <c r="J22" s="196"/>
+      <c r="K22" s="197"/>
       <c r="L22" s="14"/>
     </row>
     <row r="23" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4622,339 +4622,339 @@
       <c r="L23" s="14"/>
     </row>
     <row r="24" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="194" t="s">
+      <c r="A24" s="198" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="195"/>
-      <c r="C24" s="195"/>
-      <c r="D24" s="195"/>
-      <c r="E24" s="195"/>
-      <c r="F24" s="195"/>
-      <c r="G24" s="195"/>
-      <c r="H24" s="195"/>
-      <c r="I24" s="195"/>
-      <c r="J24" s="195"/>
-      <c r="K24" s="196"/>
+      <c r="B24" s="199"/>
+      <c r="C24" s="199"/>
+      <c r="D24" s="199"/>
+      <c r="E24" s="199"/>
+      <c r="F24" s="199"/>
+      <c r="G24" s="199"/>
+      <c r="H24" s="199"/>
+      <c r="I24" s="199"/>
+      <c r="J24" s="199"/>
+      <c r="K24" s="200"/>
       <c r="L24" s="14"/>
     </row>
     <row r="25" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="191"/>
-      <c r="B25" s="192"/>
-      <c r="C25" s="192"/>
-      <c r="D25" s="192"/>
-      <c r="E25" s="192"/>
-      <c r="F25" s="192"/>
-      <c r="G25" s="192"/>
-      <c r="H25" s="192"/>
-      <c r="I25" s="192"/>
-      <c r="J25" s="192"/>
-      <c r="K25" s="193"/>
+      <c r="A25" s="195"/>
+      <c r="B25" s="196"/>
+      <c r="C25" s="196"/>
+      <c r="D25" s="196"/>
+      <c r="E25" s="196"/>
+      <c r="F25" s="196"/>
+      <c r="G25" s="196"/>
+      <c r="H25" s="196"/>
+      <c r="I25" s="196"/>
+      <c r="J25" s="196"/>
+      <c r="K25" s="197"/>
       <c r="L25" s="14"/>
     </row>
     <row r="26" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="191"/>
-      <c r="B26" s="192"/>
-      <c r="C26" s="192"/>
-      <c r="D26" s="192"/>
-      <c r="E26" s="192"/>
-      <c r="F26" s="192"/>
-      <c r="G26" s="192"/>
-      <c r="H26" s="192"/>
-      <c r="I26" s="192"/>
-      <c r="J26" s="192"/>
-      <c r="K26" s="193"/>
+      <c r="A26" s="195"/>
+      <c r="B26" s="196"/>
+      <c r="C26" s="196"/>
+      <c r="D26" s="196"/>
+      <c r="E26" s="196"/>
+      <c r="F26" s="196"/>
+      <c r="G26" s="196"/>
+      <c r="H26" s="196"/>
+      <c r="I26" s="196"/>
+      <c r="J26" s="196"/>
+      <c r="K26" s="197"/>
       <c r="L26" s="14"/>
     </row>
     <row r="27" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="191"/>
-      <c r="B27" s="192"/>
-      <c r="C27" s="192"/>
-      <c r="D27" s="192"/>
-      <c r="E27" s="192"/>
-      <c r="F27" s="192"/>
-      <c r="G27" s="192"/>
-      <c r="H27" s="192"/>
-      <c r="I27" s="192"/>
-      <c r="J27" s="192"/>
-      <c r="K27" s="193"/>
+      <c r="A27" s="195"/>
+      <c r="B27" s="196"/>
+      <c r="C27" s="196"/>
+      <c r="D27" s="196"/>
+      <c r="E27" s="196"/>
+      <c r="F27" s="196"/>
+      <c r="G27" s="196"/>
+      <c r="H27" s="196"/>
+      <c r="I27" s="196"/>
+      <c r="J27" s="196"/>
+      <c r="K27" s="197"/>
       <c r="L27" s="14"/>
     </row>
     <row r="28" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="191"/>
-      <c r="B28" s="192"/>
-      <c r="C28" s="192"/>
-      <c r="D28" s="192"/>
-      <c r="E28" s="192"/>
-      <c r="F28" s="192"/>
-      <c r="G28" s="192"/>
-      <c r="H28" s="192"/>
-      <c r="I28" s="192"/>
-      <c r="J28" s="192"/>
-      <c r="K28" s="193"/>
+      <c r="A28" s="195"/>
+      <c r="B28" s="196"/>
+      <c r="C28" s="196"/>
+      <c r="D28" s="196"/>
+      <c r="E28" s="196"/>
+      <c r="F28" s="196"/>
+      <c r="G28" s="196"/>
+      <c r="H28" s="196"/>
+      <c r="I28" s="196"/>
+      <c r="J28" s="196"/>
+      <c r="K28" s="197"/>
       <c r="L28" s="14"/>
     </row>
     <row r="29" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="191"/>
-      <c r="B29" s="192"/>
-      <c r="C29" s="192"/>
-      <c r="D29" s="192"/>
-      <c r="E29" s="192"/>
-      <c r="F29" s="192"/>
-      <c r="G29" s="192"/>
-      <c r="H29" s="192"/>
-      <c r="I29" s="192"/>
-      <c r="J29" s="192"/>
-      <c r="K29" s="193"/>
+      <c r="A29" s="195"/>
+      <c r="B29" s="196"/>
+      <c r="C29" s="196"/>
+      <c r="D29" s="196"/>
+      <c r="E29" s="196"/>
+      <c r="F29" s="196"/>
+      <c r="G29" s="196"/>
+      <c r="H29" s="196"/>
+      <c r="I29" s="196"/>
+      <c r="J29" s="196"/>
+      <c r="K29" s="197"/>
       <c r="L29" s="14"/>
     </row>
     <row r="30" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="191"/>
-      <c r="B30" s="192"/>
-      <c r="C30" s="192"/>
-      <c r="D30" s="192"/>
-      <c r="E30" s="192"/>
-      <c r="F30" s="192"/>
-      <c r="G30" s="192"/>
-      <c r="H30" s="192"/>
-      <c r="I30" s="192"/>
-      <c r="J30" s="192"/>
-      <c r="K30" s="193"/>
+      <c r="A30" s="195"/>
+      <c r="B30" s="196"/>
+      <c r="C30" s="196"/>
+      <c r="D30" s="196"/>
+      <c r="E30" s="196"/>
+      <c r="F30" s="196"/>
+      <c r="G30" s="196"/>
+      <c r="H30" s="196"/>
+      <c r="I30" s="196"/>
+      <c r="J30" s="196"/>
+      <c r="K30" s="197"/>
       <c r="L30" s="14"/>
     </row>
     <row r="31" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="194" t="s">
+      <c r="A31" s="198" t="s">
         <v>51</v>
       </c>
-      <c r="B31" s="195"/>
-      <c r="C31" s="195"/>
-      <c r="D31" s="195"/>
-      <c r="E31" s="195"/>
-      <c r="F31" s="195"/>
-      <c r="G31" s="195"/>
-      <c r="H31" s="195"/>
-      <c r="I31" s="195"/>
-      <c r="J31" s="195"/>
-      <c r="K31" s="195"/>
+      <c r="B31" s="199"/>
+      <c r="C31" s="199"/>
+      <c r="D31" s="199"/>
+      <c r="E31" s="199"/>
+      <c r="F31" s="199"/>
+      <c r="G31" s="199"/>
+      <c r="H31" s="199"/>
+      <c r="I31" s="199"/>
+      <c r="J31" s="199"/>
+      <c r="K31" s="199"/>
       <c r="L31" s="14"/>
     </row>
     <row r="32" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="61"/>
-      <c r="B32" s="192" t="s">
+      <c r="B32" s="196" t="s">
         <v>52</v>
       </c>
-      <c r="C32" s="192"/>
-      <c r="D32" s="192"/>
-      <c r="E32" s="192"/>
-      <c r="F32" s="192"/>
-      <c r="G32" s="192"/>
-      <c r="H32" s="192" t="s">
+      <c r="C32" s="196"/>
+      <c r="D32" s="196"/>
+      <c r="E32" s="196"/>
+      <c r="F32" s="196"/>
+      <c r="G32" s="196"/>
+      <c r="H32" s="196" t="s">
         <v>53</v>
       </c>
-      <c r="I32" s="192"/>
-      <c r="J32" s="192"/>
+      <c r="I32" s="196"/>
+      <c r="J32" s="196"/>
       <c r="K32" s="66"/>
       <c r="L32" s="14"/>
     </row>
     <row r="33" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="191"/>
-      <c r="B33" s="192"/>
-      <c r="C33" s="192"/>
-      <c r="D33" s="192"/>
-      <c r="E33" s="192"/>
-      <c r="F33" s="192"/>
-      <c r="G33" s="192"/>
-      <c r="H33" s="192"/>
-      <c r="I33" s="192"/>
-      <c r="J33" s="192"/>
-      <c r="K33" s="193"/>
+      <c r="A33" s="195"/>
+      <c r="B33" s="196"/>
+      <c r="C33" s="196"/>
+      <c r="D33" s="196"/>
+      <c r="E33" s="196"/>
+      <c r="F33" s="196"/>
+      <c r="G33" s="196"/>
+      <c r="H33" s="196"/>
+      <c r="I33" s="196"/>
+      <c r="J33" s="196"/>
+      <c r="K33" s="197"/>
       <c r="L33" s="14"/>
     </row>
     <row r="34" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="191"/>
-      <c r="B34" s="192"/>
-      <c r="C34" s="192"/>
-      <c r="D34" s="192"/>
-      <c r="E34" s="192"/>
-      <c r="F34" s="192"/>
-      <c r="G34" s="192"/>
-      <c r="H34" s="192"/>
-      <c r="I34" s="192"/>
-      <c r="J34" s="192"/>
-      <c r="K34" s="193"/>
+      <c r="A34" s="195"/>
+      <c r="B34" s="196"/>
+      <c r="C34" s="196"/>
+      <c r="D34" s="196"/>
+      <c r="E34" s="196"/>
+      <c r="F34" s="196"/>
+      <c r="G34" s="196"/>
+      <c r="H34" s="196"/>
+      <c r="I34" s="196"/>
+      <c r="J34" s="196"/>
+      <c r="K34" s="197"/>
       <c r="L34" s="14"/>
     </row>
     <row r="35" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="191"/>
-      <c r="B35" s="192"/>
-      <c r="C35" s="192"/>
-      <c r="D35" s="192"/>
-      <c r="E35" s="192"/>
-      <c r="F35" s="192"/>
-      <c r="G35" s="192"/>
-      <c r="H35" s="192"/>
-      <c r="I35" s="192"/>
-      <c r="J35" s="192"/>
-      <c r="K35" s="193"/>
+      <c r="A35" s="195"/>
+      <c r="B35" s="196"/>
+      <c r="C35" s="196"/>
+      <c r="D35" s="196"/>
+      <c r="E35" s="196"/>
+      <c r="F35" s="196"/>
+      <c r="G35" s="196"/>
+      <c r="H35" s="196"/>
+      <c r="I35" s="196"/>
+      <c r="J35" s="196"/>
+      <c r="K35" s="197"/>
       <c r="L35" s="14"/>
     </row>
     <row r="36" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="191"/>
-      <c r="B36" s="192"/>
-      <c r="C36" s="192"/>
-      <c r="D36" s="192"/>
-      <c r="E36" s="192"/>
-      <c r="F36" s="192"/>
-      <c r="G36" s="192"/>
-      <c r="H36" s="192"/>
-      <c r="I36" s="192"/>
-      <c r="J36" s="192"/>
-      <c r="K36" s="193"/>
+      <c r="A36" s="195"/>
+      <c r="B36" s="196"/>
+      <c r="C36" s="196"/>
+      <c r="D36" s="196"/>
+      <c r="E36" s="196"/>
+      <c r="F36" s="196"/>
+      <c r="G36" s="196"/>
+      <c r="H36" s="196"/>
+      <c r="I36" s="196"/>
+      <c r="J36" s="196"/>
+      <c r="K36" s="197"/>
       <c r="L36" s="14"/>
     </row>
     <row r="37" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="191"/>
-      <c r="B37" s="192"/>
-      <c r="C37" s="192"/>
-      <c r="D37" s="192"/>
-      <c r="E37" s="192"/>
-      <c r="F37" s="192"/>
-      <c r="G37" s="192"/>
-      <c r="H37" s="192"/>
-      <c r="I37" s="192"/>
-      <c r="J37" s="192"/>
-      <c r="K37" s="193"/>
+      <c r="A37" s="195"/>
+      <c r="B37" s="196"/>
+      <c r="C37" s="196"/>
+      <c r="D37" s="196"/>
+      <c r="E37" s="196"/>
+      <c r="F37" s="196"/>
+      <c r="G37" s="196"/>
+      <c r="H37" s="196"/>
+      <c r="I37" s="196"/>
+      <c r="J37" s="196"/>
+      <c r="K37" s="197"/>
       <c r="L37" s="14"/>
     </row>
     <row r="38" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="191"/>
-      <c r="B38" s="192"/>
-      <c r="C38" s="192"/>
-      <c r="D38" s="192"/>
-      <c r="E38" s="192"/>
-      <c r="F38" s="192"/>
-      <c r="G38" s="192"/>
-      <c r="H38" s="192"/>
-      <c r="I38" s="192"/>
-      <c r="J38" s="192"/>
-      <c r="K38" s="193"/>
+      <c r="A38" s="195"/>
+      <c r="B38" s="196"/>
+      <c r="C38" s="196"/>
+      <c r="D38" s="196"/>
+      <c r="E38" s="196"/>
+      <c r="F38" s="196"/>
+      <c r="G38" s="196"/>
+      <c r="H38" s="196"/>
+      <c r="I38" s="196"/>
+      <c r="J38" s="196"/>
+      <c r="K38" s="197"/>
       <c r="L38" s="14"/>
     </row>
     <row r="39" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="191"/>
-      <c r="B39" s="192"/>
-      <c r="C39" s="192"/>
-      <c r="D39" s="192"/>
-      <c r="E39" s="192"/>
-      <c r="F39" s="192"/>
-      <c r="G39" s="192"/>
-      <c r="H39" s="192"/>
-      <c r="I39" s="192"/>
-      <c r="J39" s="192"/>
-      <c r="K39" s="193"/>
+      <c r="A39" s="195"/>
+      <c r="B39" s="196"/>
+      <c r="C39" s="196"/>
+      <c r="D39" s="196"/>
+      <c r="E39" s="196"/>
+      <c r="F39" s="196"/>
+      <c r="G39" s="196"/>
+      <c r="H39" s="196"/>
+      <c r="I39" s="196"/>
+      <c r="J39" s="196"/>
+      <c r="K39" s="197"/>
       <c r="L39" s="14"/>
     </row>
     <row r="40" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="191"/>
-      <c r="B40" s="192"/>
-      <c r="C40" s="192"/>
-      <c r="D40" s="192"/>
-      <c r="E40" s="192"/>
-      <c r="F40" s="192"/>
-      <c r="G40" s="192"/>
-      <c r="H40" s="192"/>
-      <c r="I40" s="192"/>
-      <c r="J40" s="192"/>
-      <c r="K40" s="193"/>
+      <c r="A40" s="195"/>
+      <c r="B40" s="196"/>
+      <c r="C40" s="196"/>
+      <c r="D40" s="196"/>
+      <c r="E40" s="196"/>
+      <c r="F40" s="196"/>
+      <c r="G40" s="196"/>
+      <c r="H40" s="196"/>
+      <c r="I40" s="196"/>
+      <c r="J40" s="196"/>
+      <c r="K40" s="197"/>
       <c r="L40" s="14"/>
     </row>
     <row r="41" spans="1:12" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="197" t="s">
+      <c r="A41" s="201" t="s">
         <v>54</v>
       </c>
-      <c r="B41" s="198"/>
-      <c r="C41" s="198"/>
-      <c r="D41" s="198"/>
-      <c r="E41" s="198"/>
-      <c r="F41" s="198"/>
-      <c r="G41" s="198"/>
-      <c r="H41" s="192"/>
-      <c r="I41" s="192"/>
-      <c r="J41" s="192"/>
-      <c r="K41" s="193"/>
+      <c r="B41" s="202"/>
+      <c r="C41" s="202"/>
+      <c r="D41" s="202"/>
+      <c r="E41" s="202"/>
+      <c r="F41" s="202"/>
+      <c r="G41" s="202"/>
+      <c r="H41" s="196"/>
+      <c r="I41" s="196"/>
+      <c r="J41" s="196"/>
+      <c r="K41" s="197"/>
       <c r="L41" s="14"/>
     </row>
     <row r="42" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="194" t="s">
+      <c r="A42" s="198" t="s">
         <v>55</v>
       </c>
-      <c r="B42" s="195"/>
-      <c r="C42" s="195"/>
-      <c r="D42" s="195"/>
-      <c r="E42" s="195"/>
-      <c r="F42" s="195"/>
-      <c r="G42" s="195"/>
-      <c r="H42" s="195"/>
-      <c r="I42" s="195"/>
-      <c r="J42" s="195"/>
-      <c r="K42" s="196"/>
+      <c r="B42" s="199"/>
+      <c r="C42" s="199"/>
+      <c r="D42" s="199"/>
+      <c r="E42" s="199"/>
+      <c r="F42" s="199"/>
+      <c r="G42" s="199"/>
+      <c r="H42" s="199"/>
+      <c r="I42" s="199"/>
+      <c r="J42" s="199"/>
+      <c r="K42" s="200"/>
       <c r="L42" s="14"/>
     </row>
     <row r="43" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="191"/>
-      <c r="B43" s="192"/>
-      <c r="C43" s="192"/>
-      <c r="D43" s="192"/>
-      <c r="E43" s="192"/>
-      <c r="F43" s="192"/>
-      <c r="G43" s="192"/>
-      <c r="H43" s="192"/>
-      <c r="I43" s="192"/>
-      <c r="J43" s="192"/>
-      <c r="K43" s="193"/>
+      <c r="A43" s="195"/>
+      <c r="B43" s="196"/>
+      <c r="C43" s="196"/>
+      <c r="D43" s="196"/>
+      <c r="E43" s="196"/>
+      <c r="F43" s="196"/>
+      <c r="G43" s="196"/>
+      <c r="H43" s="196"/>
+      <c r="I43" s="196"/>
+      <c r="J43" s="196"/>
+      <c r="K43" s="197"/>
       <c r="L43" s="14"/>
     </row>
     <row r="44" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="191"/>
-      <c r="B44" s="192"/>
-      <c r="C44" s="192"/>
-      <c r="D44" s="192"/>
-      <c r="E44" s="192"/>
-      <c r="F44" s="192"/>
-      <c r="G44" s="192"/>
-      <c r="H44" s="192"/>
-      <c r="I44" s="192"/>
-      <c r="J44" s="192"/>
-      <c r="K44" s="193"/>
+      <c r="A44" s="195"/>
+      <c r="B44" s="196"/>
+      <c r="C44" s="196"/>
+      <c r="D44" s="196"/>
+      <c r="E44" s="196"/>
+      <c r="F44" s="196"/>
+      <c r="G44" s="196"/>
+      <c r="H44" s="196"/>
+      <c r="I44" s="196"/>
+      <c r="J44" s="196"/>
+      <c r="K44" s="197"/>
       <c r="L44" s="14"/>
     </row>
     <row r="45" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="191"/>
-      <c r="B45" s="192"/>
-      <c r="C45" s="192"/>
-      <c r="D45" s="192"/>
-      <c r="E45" s="192"/>
-      <c r="F45" s="192"/>
-      <c r="G45" s="192"/>
-      <c r="H45" s="192"/>
-      <c r="I45" s="192"/>
-      <c r="J45" s="192"/>
-      <c r="K45" s="193"/>
+      <c r="A45" s="195"/>
+      <c r="B45" s="196"/>
+      <c r="C45" s="196"/>
+      <c r="D45" s="196"/>
+      <c r="E45" s="196"/>
+      <c r="F45" s="196"/>
+      <c r="G45" s="196"/>
+      <c r="H45" s="196"/>
+      <c r="I45" s="196"/>
+      <c r="J45" s="196"/>
+      <c r="K45" s="197"/>
       <c r="L45" s="14"/>
     </row>
     <row r="46" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="194" t="s">
+      <c r="A46" s="198" t="s">
         <v>56</v>
       </c>
-      <c r="B46" s="195"/>
-      <c r="C46" s="195"/>
-      <c r="D46" s="195"/>
-      <c r="E46" s="195"/>
-      <c r="F46" s="195"/>
-      <c r="G46" s="195"/>
-      <c r="H46" s="195"/>
-      <c r="I46" s="195"/>
-      <c r="J46" s="195"/>
-      <c r="K46" s="195"/>
+      <c r="B46" s="199"/>
+      <c r="C46" s="199"/>
+      <c r="D46" s="199"/>
+      <c r="E46" s="199"/>
+      <c r="F46" s="199"/>
+      <c r="G46" s="199"/>
+      <c r="H46" s="199"/>
+      <c r="I46" s="199"/>
+      <c r="J46" s="199"/>
+      <c r="K46" s="199"/>
       <c r="L46" s="14"/>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
@@ -4973,12 +4973,12 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="32"/>
-      <c r="B48" s="161"/>
-      <c r="C48" s="161"/>
-      <c r="D48" s="161"/>
-      <c r="E48" s="161"/>
-      <c r="F48" s="161"/>
-      <c r="G48" s="161"/>
+      <c r="B48" s="165"/>
+      <c r="C48" s="165"/>
+      <c r="D48" s="165"/>
+      <c r="E48" s="165"/>
+      <c r="F48" s="165"/>
+      <c r="G48" s="165"/>
       <c r="H48" s="33"/>
       <c r="I48" s="33"/>
       <c r="J48" s="33"/>
@@ -5044,36 +5044,36 @@
     <row r="53" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="35"/>
       <c r="B53" s="36"/>
-      <c r="C53" s="157" t="s">
+      <c r="C53" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="D53" s="157"/>
-      <c r="E53" s="157"/>
-      <c r="F53" s="157"/>
+      <c r="D53" s="161"/>
+      <c r="E53" s="161"/>
+      <c r="F53" s="161"/>
       <c r="G53" s="38"/>
-      <c r="H53" s="157" t="s">
+      <c r="H53" s="161" t="s">
         <v>29</v>
       </c>
-      <c r="I53" s="157"/>
-      <c r="J53" s="157"/>
+      <c r="I53" s="161"/>
+      <c r="J53" s="161"/>
       <c r="K53" s="39"/>
       <c r="L53" s="14"/>
     </row>
     <row r="54" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="35"/>
       <c r="B54" s="36"/>
-      <c r="C54" s="158" t="s">
+      <c r="C54" s="162" t="s">
         <v>30</v>
       </c>
-      <c r="D54" s="158"/>
-      <c r="E54" s="158"/>
-      <c r="F54" s="158"/>
+      <c r="D54" s="162"/>
+      <c r="E54" s="162"/>
+      <c r="F54" s="162"/>
       <c r="G54" s="38"/>
-      <c r="H54" s="158" t="s">
+      <c r="H54" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="I54" s="158"/>
-      <c r="J54" s="158"/>
+      <c r="I54" s="162"/>
+      <c r="J54" s="162"/>
       <c r="K54" s="39"/>
       <c r="L54" s="14"/>
     </row>
@@ -5085,11 +5085,11 @@
       <c r="E55" s="38"/>
       <c r="F55" s="38"/>
       <c r="G55" s="38"/>
-      <c r="H55" s="162" t="s">
+      <c r="H55" s="166" t="s">
         <v>32</v>
       </c>
-      <c r="I55" s="162"/>
-      <c r="J55" s="162"/>
+      <c r="I55" s="166"/>
+      <c r="J55" s="166"/>
       <c r="K55" s="39"/>
       <c r="L55" s="14"/>
     </row>
@@ -5108,35 +5108,35 @@
       <c r="L56" s="14"/>
     </row>
     <row r="57" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="130" t="s">
+      <c r="A57" s="134" t="s">
         <v>33</v>
       </c>
-      <c r="B57" s="131"/>
-      <c r="C57" s="131"/>
-      <c r="D57" s="131"/>
-      <c r="E57" s="131"/>
-      <c r="F57" s="131"/>
-      <c r="G57" s="131"/>
-      <c r="H57" s="131"/>
-      <c r="I57" s="131"/>
-      <c r="J57" s="131"/>
-      <c r="K57" s="132"/>
+      <c r="B57" s="135"/>
+      <c r="C57" s="135"/>
+      <c r="D57" s="135"/>
+      <c r="E57" s="135"/>
+      <c r="F57" s="135"/>
+      <c r="G57" s="135"/>
+      <c r="H57" s="135"/>
+      <c r="I57" s="135"/>
+      <c r="J57" s="135"/>
+      <c r="K57" s="136"/>
       <c r="L57" s="14"/>
     </row>
     <row r="58" spans="1:12" ht="86.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="133" t="s">
+      <c r="A58" s="137" t="s">
         <v>57</v>
       </c>
-      <c r="B58" s="134"/>
-      <c r="C58" s="134"/>
-      <c r="D58" s="134"/>
-      <c r="E58" s="134"/>
-      <c r="F58" s="134"/>
-      <c r="G58" s="134"/>
-      <c r="H58" s="134"/>
-      <c r="I58" s="134"/>
-      <c r="J58" s="134"/>
-      <c r="K58" s="135"/>
+      <c r="B58" s="138"/>
+      <c r="C58" s="138"/>
+      <c r="D58" s="138"/>
+      <c r="E58" s="138"/>
+      <c r="F58" s="138"/>
+      <c r="G58" s="138"/>
+      <c r="H58" s="138"/>
+      <c r="I58" s="138"/>
+      <c r="J58" s="138"/>
+      <c r="K58" s="139"/>
       <c r="L58" s="14"/>
     </row>
   </sheetData>
@@ -5212,63 +5212,63 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E2" s="203" t="s">
+      <c r="E2" s="207" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="203"/>
-      <c r="G2" s="203"/>
-      <c r="H2" s="203"/>
-      <c r="I2" s="203"/>
-      <c r="J2" s="203"/>
+      <c r="F2" s="207"/>
+      <c r="G2" s="207"/>
+      <c r="H2" s="207"/>
+      <c r="I2" s="207"/>
+      <c r="J2" s="207"/>
     </row>
     <row r="3" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E3" s="204" t="s">
+      <c r="E3" s="208" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="204"/>
-      <c r="G3" s="204"/>
-      <c r="H3" s="204"/>
-      <c r="I3" s="204"/>
-      <c r="J3" s="204"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="208"/>
+      <c r="H3" s="208"/>
+      <c r="I3" s="208"/>
+      <c r="J3" s="208"/>
     </row>
     <row r="4" spans="2:14" ht="4.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:14" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="205" t="s">
+      <c r="B5" s="209" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="206"/>
-      <c r="D5" s="206"/>
-      <c r="E5" s="206"/>
-      <c r="F5" s="206"/>
-      <c r="G5" s="206"/>
-      <c r="H5" s="206"/>
-      <c r="I5" s="206"/>
-      <c r="J5" s="206"/>
-      <c r="K5" s="206"/>
-      <c r="L5" s="206"/>
-      <c r="M5" s="206"/>
-      <c r="N5" s="207"/>
+      <c r="C5" s="210"/>
+      <c r="D5" s="210"/>
+      <c r="E5" s="210"/>
+      <c r="F5" s="210"/>
+      <c r="G5" s="210"/>
+      <c r="H5" s="210"/>
+      <c r="I5" s="210"/>
+      <c r="J5" s="210"/>
+      <c r="K5" s="210"/>
+      <c r="L5" s="210"/>
+      <c r="M5" s="210"/>
+      <c r="N5" s="211"/>
     </row>
     <row r="6" spans="2:14" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="75"/>
       <c r="N6" s="74"/>
     </row>
     <row r="7" spans="2:14" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="208" t="s">
+      <c r="B7" s="212" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="209"/>
+      <c r="C7" s="213"/>
       <c r="D7" s="99"/>
-      <c r="E7" s="210"/>
-      <c r="F7" s="210"/>
-      <c r="G7" s="210"/>
+      <c r="E7" s="214"/>
+      <c r="F7" s="214"/>
+      <c r="G7" s="214"/>
       <c r="H7" s="90"/>
       <c r="I7" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="J7" s="211"/>
-      <c r="K7" s="211"/>
-      <c r="L7" s="211"/>
+      <c r="J7" s="215"/>
+      <c r="K7" s="215"/>
+      <c r="L7" s="215"/>
       <c r="M7" s="90"/>
       <c r="N7" s="80"/>
     </row>
@@ -5277,21 +5277,21 @@
       <c r="N8" s="74"/>
     </row>
     <row r="9" spans="2:14" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="208" t="s">
+      <c r="B9" s="212" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="209"/>
+      <c r="C9" s="213"/>
       <c r="D9" s="99"/>
-      <c r="E9" s="210"/>
-      <c r="F9" s="210"/>
-      <c r="G9" s="210"/>
+      <c r="E9" s="214"/>
+      <c r="F9" s="214"/>
+      <c r="G9" s="214"/>
       <c r="H9" s="90"/>
       <c r="I9" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="J9" s="211"/>
-      <c r="K9" s="215"/>
-      <c r="L9" s="215"/>
+      <c r="J9" s="215"/>
+      <c r="K9" s="219"/>
+      <c r="L9" s="219"/>
       <c r="M9" s="90"/>
       <c r="N9" s="80"/>
     </row>
@@ -5300,52 +5300,52 @@
       <c r="N10" s="74"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="216" t="s">
+      <c r="B11" s="220" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="216"/>
+      <c r="C11" s="220"/>
       <c r="D11" s="100"/>
-      <c r="E11" s="217" t="s">
+      <c r="E11" s="221" t="s">
         <v>89</v>
       </c>
-      <c r="F11" s="218"/>
-      <c r="G11" s="218"/>
-      <c r="H11" s="218"/>
-      <c r="I11" s="218"/>
-      <c r="J11" s="218"/>
-      <c r="K11" s="218"/>
-      <c r="L11" s="218"/>
-      <c r="M11" s="219"/>
+      <c r="F11" s="222"/>
+      <c r="G11" s="222"/>
+      <c r="H11" s="222"/>
+      <c r="I11" s="222"/>
+      <c r="J11" s="222"/>
+      <c r="K11" s="222"/>
+      <c r="L11" s="222"/>
+      <c r="M11" s="223"/>
       <c r="N11" s="81"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="216"/>
-      <c r="C12" s="216"/>
+      <c r="B12" s="220"/>
+      <c r="C12" s="220"/>
       <c r="D12" s="100"/>
-      <c r="E12" s="220"/>
-      <c r="F12" s="221"/>
-      <c r="G12" s="221"/>
-      <c r="H12" s="221"/>
-      <c r="I12" s="221"/>
-      <c r="J12" s="221"/>
-      <c r="K12" s="221"/>
-      <c r="L12" s="221"/>
-      <c r="M12" s="222"/>
+      <c r="E12" s="224"/>
+      <c r="F12" s="225"/>
+      <c r="G12" s="225"/>
+      <c r="H12" s="225"/>
+      <c r="I12" s="225"/>
+      <c r="J12" s="225"/>
+      <c r="K12" s="225"/>
+      <c r="L12" s="225"/>
+      <c r="M12" s="226"/>
       <c r="N12" s="81"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="216"/>
-      <c r="C13" s="216"/>
+      <c r="B13" s="220"/>
+      <c r="C13" s="220"/>
       <c r="D13" s="100"/>
-      <c r="E13" s="223"/>
-      <c r="F13" s="224"/>
-      <c r="G13" s="224"/>
-      <c r="H13" s="224"/>
-      <c r="I13" s="224"/>
-      <c r="J13" s="224"/>
-      <c r="K13" s="224"/>
-      <c r="L13" s="224"/>
-      <c r="M13" s="225"/>
+      <c r="E13" s="227"/>
+      <c r="F13" s="228"/>
+      <c r="G13" s="228"/>
+      <c r="H13" s="228"/>
+      <c r="I13" s="228"/>
+      <c r="J13" s="228"/>
+      <c r="K13" s="228"/>
+      <c r="L13" s="228"/>
+      <c r="M13" s="229"/>
       <c r="N13" s="81"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
@@ -5353,22 +5353,22 @@
       <c r="N14" s="74"/>
     </row>
     <row r="15" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="208" t="s">
+      <c r="B15" s="212" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="209"/>
+      <c r="C15" s="213"/>
       <c r="D15" s="99"/>
-      <c r="E15" s="226"/>
-      <c r="F15" s="227"/>
-      <c r="G15" s="227"/>
+      <c r="E15" s="230"/>
+      <c r="F15" s="231"/>
+      <c r="G15" s="231"/>
       <c r="H15" s="78"/>
-      <c r="I15" s="209" t="s">
+      <c r="I15" s="213" t="s">
         <v>66</v>
       </c>
-      <c r="J15" s="209"/>
-      <c r="K15" s="228"/>
-      <c r="L15" s="229"/>
-      <c r="M15" s="230"/>
+      <c r="J15" s="213"/>
+      <c r="K15" s="232"/>
+      <c r="L15" s="233"/>
+      <c r="M15" s="234"/>
       <c r="N15" s="82"/>
     </row>
     <row r="16" spans="2:14" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -5376,22 +5376,22 @@
       <c r="N16" s="74"/>
     </row>
     <row r="17" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="208" t="s">
+      <c r="B17" s="212" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="209"/>
+      <c r="C17" s="213"/>
       <c r="D17" s="99"/>
-      <c r="E17" s="227"/>
-      <c r="F17" s="227"/>
-      <c r="G17" s="227"/>
+      <c r="E17" s="231"/>
+      <c r="F17" s="231"/>
+      <c r="G17" s="231"/>
       <c r="H17" s="79"/>
-      <c r="I17" s="209" t="s">
+      <c r="I17" s="213" t="s">
         <v>68</v>
       </c>
-      <c r="J17" s="209"/>
-      <c r="K17" s="231"/>
-      <c r="L17" s="229"/>
-      <c r="M17" s="230"/>
+      <c r="J17" s="213"/>
+      <c r="K17" s="235"/>
+      <c r="L17" s="233"/>
+      <c r="M17" s="234"/>
       <c r="N17" s="82"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.3">
@@ -5410,155 +5410,155 @@
       <c r="N20" s="74"/>
     </row>
     <row r="21" spans="2:14" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="205" t="s">
+      <c r="B21" s="209" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="206"/>
-      <c r="D21" s="206"/>
-      <c r="E21" s="206"/>
-      <c r="F21" s="206"/>
-      <c r="G21" s="206"/>
-      <c r="H21" s="206"/>
-      <c r="I21" s="206"/>
-      <c r="J21" s="206"/>
-      <c r="K21" s="206"/>
-      <c r="L21" s="206"/>
-      <c r="M21" s="206"/>
-      <c r="N21" s="207"/>
+      <c r="C21" s="210"/>
+      <c r="D21" s="210"/>
+      <c r="E21" s="210"/>
+      <c r="F21" s="210"/>
+      <c r="G21" s="210"/>
+      <c r="H21" s="210"/>
+      <c r="I21" s="210"/>
+      <c r="J21" s="210"/>
+      <c r="K21" s="210"/>
+      <c r="L21" s="210"/>
+      <c r="M21" s="210"/>
+      <c r="N21" s="211"/>
     </row>
     <row r="22" spans="2:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="212" t="s">
+      <c r="B22" s="216" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="213"/>
-      <c r="D22" s="213"/>
-      <c r="E22" s="213"/>
-      <c r="F22" s="213"/>
-      <c r="G22" s="213"/>
-      <c r="H22" s="213"/>
-      <c r="I22" s="213"/>
-      <c r="J22" s="213"/>
-      <c r="K22" s="213"/>
-      <c r="L22" s="213"/>
-      <c r="M22" s="213"/>
-      <c r="N22" s="214"/>
+      <c r="C22" s="217"/>
+      <c r="D22" s="217"/>
+      <c r="E22" s="217"/>
+      <c r="F22" s="217"/>
+      <c r="G22" s="217"/>
+      <c r="H22" s="217"/>
+      <c r="I22" s="217"/>
+      <c r="J22" s="217"/>
+      <c r="K22" s="217"/>
+      <c r="L22" s="217"/>
+      <c r="M22" s="217"/>
+      <c r="N22" s="218"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B23" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="235" t="s">
+      <c r="C23" s="239" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="236"/>
-      <c r="E23" s="236"/>
-      <c r="F23" s="236"/>
-      <c r="G23" s="236"/>
-      <c r="H23" s="237"/>
-      <c r="I23" s="235" t="s">
+      <c r="D23" s="240"/>
+      <c r="E23" s="240"/>
+      <c r="F23" s="240"/>
+      <c r="G23" s="240"/>
+      <c r="H23" s="241"/>
+      <c r="I23" s="239" t="s">
         <v>73</v>
       </c>
-      <c r="J23" s="237"/>
-      <c r="K23" s="235" t="s">
+      <c r="J23" s="241"/>
+      <c r="K23" s="239" t="s">
         <v>74</v>
       </c>
-      <c r="L23" s="236"/>
-      <c r="M23" s="236"/>
-      <c r="N23" s="237"/>
+      <c r="L23" s="240"/>
+      <c r="M23" s="240"/>
+      <c r="N23" s="241"/>
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B24" s="73">
         <v>1</v>
       </c>
-      <c r="C24" s="232" t="s">
+      <c r="C24" s="236" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="233"/>
-      <c r="E24" s="233"/>
-      <c r="F24" s="233"/>
-      <c r="G24" s="233"/>
-      <c r="H24" s="234"/>
-      <c r="I24" s="232"/>
-      <c r="J24" s="234"/>
-      <c r="K24" s="232"/>
-      <c r="L24" s="233"/>
-      <c r="M24" s="233"/>
+      <c r="D24" s="237"/>
+      <c r="E24" s="237"/>
+      <c r="F24" s="237"/>
+      <c r="G24" s="237"/>
+      <c r="H24" s="238"/>
+      <c r="I24" s="236"/>
+      <c r="J24" s="238"/>
+      <c r="K24" s="236"/>
+      <c r="L24" s="237"/>
+      <c r="M24" s="237"/>
       <c r="N24" s="85"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B25" s="73">
         <v>2</v>
       </c>
-      <c r="C25" s="232" t="s">
+      <c r="C25" s="236" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="233"/>
-      <c r="E25" s="233"/>
-      <c r="F25" s="233"/>
-      <c r="G25" s="233"/>
-      <c r="H25" s="234"/>
-      <c r="I25" s="232"/>
-      <c r="J25" s="234"/>
-      <c r="K25" s="232"/>
-      <c r="L25" s="233"/>
-      <c r="M25" s="233"/>
+      <c r="D25" s="237"/>
+      <c r="E25" s="237"/>
+      <c r="F25" s="237"/>
+      <c r="G25" s="237"/>
+      <c r="H25" s="238"/>
+      <c r="I25" s="236"/>
+      <c r="J25" s="238"/>
+      <c r="K25" s="236"/>
+      <c r="L25" s="237"/>
+      <c r="M25" s="237"/>
       <c r="N25" s="86"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B26" s="73">
         <v>3</v>
       </c>
-      <c r="C26" s="232" t="s">
+      <c r="C26" s="236" t="s">
         <v>77</v>
       </c>
-      <c r="D26" s="233"/>
-      <c r="E26" s="233"/>
-      <c r="F26" s="233"/>
-      <c r="G26" s="233"/>
-      <c r="H26" s="234"/>
+      <c r="D26" s="237"/>
+      <c r="E26" s="237"/>
+      <c r="F26" s="237"/>
+      <c r="G26" s="237"/>
+      <c r="H26" s="238"/>
       <c r="I26" s="101"/>
       <c r="J26" s="102"/>
-      <c r="K26" s="232"/>
-      <c r="L26" s="233"/>
-      <c r="M26" s="233"/>
+      <c r="K26" s="236"/>
+      <c r="L26" s="237"/>
+      <c r="M26" s="237"/>
       <c r="N26" s="86"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B27" s="73">
         <v>4</v>
       </c>
-      <c r="C27" s="232" t="s">
+      <c r="C27" s="236" t="s">
         <v>78</v>
       </c>
-      <c r="D27" s="233"/>
-      <c r="E27" s="233"/>
-      <c r="F27" s="233"/>
-      <c r="G27" s="233"/>
-      <c r="H27" s="234"/>
-      <c r="I27" s="232"/>
-      <c r="J27" s="234"/>
-      <c r="K27" s="232"/>
-      <c r="L27" s="233"/>
-      <c r="M27" s="233"/>
+      <c r="D27" s="237"/>
+      <c r="E27" s="237"/>
+      <c r="F27" s="237"/>
+      <c r="G27" s="237"/>
+      <c r="H27" s="238"/>
+      <c r="I27" s="236"/>
+      <c r="J27" s="238"/>
+      <c r="K27" s="236"/>
+      <c r="L27" s="237"/>
+      <c r="M27" s="237"/>
       <c r="N27" s="86"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B28" s="73">
         <v>5</v>
       </c>
-      <c r="C28" s="232" t="s">
+      <c r="C28" s="236" t="s">
         <v>79</v>
       </c>
-      <c r="D28" s="233"/>
-      <c r="E28" s="233"/>
-      <c r="F28" s="233"/>
-      <c r="G28" s="233"/>
-      <c r="H28" s="234"/>
-      <c r="I28" s="232"/>
-      <c r="J28" s="234"/>
-      <c r="K28" s="232"/>
-      <c r="L28" s="233"/>
-      <c r="M28" s="233"/>
+      <c r="D28" s="237"/>
+      <c r="E28" s="237"/>
+      <c r="F28" s="237"/>
+      <c r="G28" s="237"/>
+      <c r="H28" s="238"/>
+      <c r="I28" s="236"/>
+      <c r="J28" s="238"/>
+      <c r="K28" s="236"/>
+      <c r="L28" s="237"/>
+      <c r="M28" s="237"/>
       <c r="N28" s="86"/>
     </row>
     <row r="29" spans="2:14" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -5566,95 +5566,95 @@
       <c r="N29" s="74"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B30" s="241" t="s">
+      <c r="B30" s="245" t="s">
         <v>80</v>
       </c>
-      <c r="C30" s="242"/>
-      <c r="D30" s="242"/>
-      <c r="E30" s="242"/>
-      <c r="F30" s="242"/>
-      <c r="G30" s="242"/>
-      <c r="H30" s="242"/>
-      <c r="I30" s="242"/>
-      <c r="J30" s="242"/>
-      <c r="K30" s="242"/>
-      <c r="L30" s="242"/>
-      <c r="M30" s="242"/>
-      <c r="N30" s="243"/>
+      <c r="C30" s="246"/>
+      <c r="D30" s="246"/>
+      <c r="E30" s="246"/>
+      <c r="F30" s="246"/>
+      <c r="G30" s="246"/>
+      <c r="H30" s="246"/>
+      <c r="I30" s="246"/>
+      <c r="J30" s="246"/>
+      <c r="K30" s="246"/>
+      <c r="L30" s="246"/>
+      <c r="M30" s="246"/>
+      <c r="N30" s="247"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B31" s="244"/>
-      <c r="C31" s="245"/>
-      <c r="D31" s="245"/>
-      <c r="E31" s="245"/>
-      <c r="F31" s="245"/>
-      <c r="G31" s="245"/>
-      <c r="H31" s="245"/>
-      <c r="I31" s="245"/>
-      <c r="J31" s="245"/>
-      <c r="K31" s="245"/>
-      <c r="L31" s="245"/>
-      <c r="M31" s="245"/>
+      <c r="B31" s="248"/>
+      <c r="C31" s="249"/>
+      <c r="D31" s="249"/>
+      <c r="E31" s="249"/>
+      <c r="F31" s="249"/>
+      <c r="G31" s="249"/>
+      <c r="H31" s="249"/>
+      <c r="I31" s="249"/>
+      <c r="J31" s="249"/>
+      <c r="K31" s="249"/>
+      <c r="L31" s="249"/>
+      <c r="M31" s="249"/>
       <c r="N31" s="84"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B32" s="244"/>
-      <c r="C32" s="245"/>
-      <c r="D32" s="245"/>
-      <c r="E32" s="245"/>
-      <c r="F32" s="245"/>
-      <c r="G32" s="245"/>
-      <c r="H32" s="245"/>
-      <c r="I32" s="245"/>
-      <c r="J32" s="245"/>
-      <c r="K32" s="245"/>
-      <c r="L32" s="245"/>
-      <c r="M32" s="245"/>
+      <c r="B32" s="248"/>
+      <c r="C32" s="249"/>
+      <c r="D32" s="249"/>
+      <c r="E32" s="249"/>
+      <c r="F32" s="249"/>
+      <c r="G32" s="249"/>
+      <c r="H32" s="249"/>
+      <c r="I32" s="249"/>
+      <c r="J32" s="249"/>
+      <c r="K32" s="249"/>
+      <c r="L32" s="249"/>
+      <c r="M32" s="249"/>
       <c r="N32" s="82"/>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B33" s="244"/>
-      <c r="C33" s="245"/>
-      <c r="D33" s="245"/>
-      <c r="E33" s="245"/>
-      <c r="F33" s="245"/>
-      <c r="G33" s="245"/>
-      <c r="H33" s="245"/>
-      <c r="I33" s="245"/>
-      <c r="J33" s="245"/>
-      <c r="K33" s="245"/>
-      <c r="L33" s="245"/>
-      <c r="M33" s="245"/>
+      <c r="B33" s="248"/>
+      <c r="C33" s="249"/>
+      <c r="D33" s="249"/>
+      <c r="E33" s="249"/>
+      <c r="F33" s="249"/>
+      <c r="G33" s="249"/>
+      <c r="H33" s="249"/>
+      <c r="I33" s="249"/>
+      <c r="J33" s="249"/>
+      <c r="K33" s="249"/>
+      <c r="L33" s="249"/>
+      <c r="M33" s="249"/>
       <c r="N33" s="82"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B34" s="244"/>
-      <c r="C34" s="245"/>
-      <c r="D34" s="245"/>
-      <c r="E34" s="245"/>
-      <c r="F34" s="245"/>
-      <c r="G34" s="245"/>
-      <c r="H34" s="245"/>
-      <c r="I34" s="245"/>
-      <c r="J34" s="245"/>
-      <c r="K34" s="245"/>
-      <c r="L34" s="245"/>
-      <c r="M34" s="245"/>
+      <c r="B34" s="248"/>
+      <c r="C34" s="249"/>
+      <c r="D34" s="249"/>
+      <c r="E34" s="249"/>
+      <c r="F34" s="249"/>
+      <c r="G34" s="249"/>
+      <c r="H34" s="249"/>
+      <c r="I34" s="249"/>
+      <c r="J34" s="249"/>
+      <c r="K34" s="249"/>
+      <c r="L34" s="249"/>
+      <c r="M34" s="249"/>
       <c r="N34" s="82"/>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B35" s="244"/>
-      <c r="C35" s="245"/>
-      <c r="D35" s="245"/>
-      <c r="E35" s="245"/>
-      <c r="F35" s="245"/>
-      <c r="G35" s="245"/>
-      <c r="H35" s="245"/>
-      <c r="I35" s="245"/>
-      <c r="J35" s="245"/>
-      <c r="K35" s="245"/>
-      <c r="L35" s="245"/>
-      <c r="M35" s="245"/>
+      <c r="B35" s="248"/>
+      <c r="C35" s="249"/>
+      <c r="D35" s="249"/>
+      <c r="E35" s="249"/>
+      <c r="F35" s="249"/>
+      <c r="G35" s="249"/>
+      <c r="H35" s="249"/>
+      <c r="I35" s="249"/>
+      <c r="J35" s="249"/>
+      <c r="K35" s="249"/>
+      <c r="L35" s="249"/>
+      <c r="M35" s="249"/>
       <c r="N35" s="82"/>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.3">
@@ -5748,18 +5748,18 @@
       <c r="N41" s="82"/>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B42" s="244"/>
-      <c r="C42" s="245"/>
-      <c r="D42" s="245"/>
-      <c r="E42" s="245"/>
-      <c r="F42" s="245"/>
-      <c r="G42" s="245"/>
-      <c r="H42" s="245"/>
-      <c r="I42" s="245"/>
-      <c r="J42" s="245"/>
-      <c r="K42" s="245"/>
-      <c r="L42" s="245"/>
-      <c r="M42" s="245"/>
+      <c r="B42" s="248"/>
+      <c r="C42" s="249"/>
+      <c r="D42" s="249"/>
+      <c r="E42" s="249"/>
+      <c r="F42" s="249"/>
+      <c r="G42" s="249"/>
+      <c r="H42" s="249"/>
+      <c r="I42" s="249"/>
+      <c r="J42" s="249"/>
+      <c r="K42" s="249"/>
+      <c r="L42" s="249"/>
+      <c r="M42" s="249"/>
       <c r="N42" s="82"/>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.3">
@@ -5782,131 +5782,131 @@
       <c r="N44" s="74"/>
     </row>
     <row r="45" spans="2:14" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B45" s="205" t="s">
+      <c r="B45" s="209" t="s">
         <v>81</v>
       </c>
-      <c r="C45" s="206"/>
-      <c r="D45" s="206"/>
-      <c r="E45" s="206"/>
-      <c r="F45" s="206"/>
-      <c r="G45" s="206"/>
-      <c r="H45" s="206"/>
-      <c r="I45" s="206"/>
-      <c r="J45" s="206"/>
-      <c r="K45" s="206"/>
-      <c r="L45" s="206"/>
-      <c r="M45" s="206"/>
-      <c r="N45" s="207"/>
+      <c r="C45" s="210"/>
+      <c r="D45" s="210"/>
+      <c r="E45" s="210"/>
+      <c r="F45" s="210"/>
+      <c r="G45" s="210"/>
+      <c r="H45" s="210"/>
+      <c r="I45" s="210"/>
+      <c r="J45" s="210"/>
+      <c r="K45" s="210"/>
+      <c r="L45" s="210"/>
+      <c r="M45" s="210"/>
+      <c r="N45" s="211"/>
     </row>
     <row r="46" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="238" t="s">
+      <c r="B46" s="242" t="s">
         <v>34</v>
       </c>
-      <c r="C46" s="239"/>
-      <c r="D46" s="239"/>
-      <c r="E46" s="239"/>
-      <c r="F46" s="239"/>
-      <c r="G46" s="239"/>
-      <c r="H46" s="239"/>
-      <c r="I46" s="239"/>
-      <c r="J46" s="239"/>
-      <c r="K46" s="239"/>
-      <c r="L46" s="239"/>
-      <c r="M46" s="239"/>
-      <c r="N46" s="240"/>
+      <c r="C46" s="243"/>
+      <c r="D46" s="243"/>
+      <c r="E46" s="243"/>
+      <c r="F46" s="243"/>
+      <c r="G46" s="243"/>
+      <c r="H46" s="243"/>
+      <c r="I46" s="243"/>
+      <c r="J46" s="243"/>
+      <c r="K46" s="243"/>
+      <c r="L46" s="243"/>
+      <c r="M46" s="243"/>
+      <c r="N46" s="244"/>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B47" s="238"/>
-      <c r="C47" s="239"/>
-      <c r="D47" s="239"/>
-      <c r="E47" s="239"/>
-      <c r="F47" s="239"/>
-      <c r="G47" s="239"/>
-      <c r="H47" s="239"/>
-      <c r="I47" s="239"/>
-      <c r="J47" s="239"/>
-      <c r="K47" s="239"/>
-      <c r="L47" s="239"/>
-      <c r="M47" s="239"/>
-      <c r="N47" s="240"/>
+      <c r="B47" s="242"/>
+      <c r="C47" s="243"/>
+      <c r="D47" s="243"/>
+      <c r="E47" s="243"/>
+      <c r="F47" s="243"/>
+      <c r="G47" s="243"/>
+      <c r="H47" s="243"/>
+      <c r="I47" s="243"/>
+      <c r="J47" s="243"/>
+      <c r="K47" s="243"/>
+      <c r="L47" s="243"/>
+      <c r="M47" s="243"/>
+      <c r="N47" s="244"/>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B48" s="238"/>
-      <c r="C48" s="239"/>
-      <c r="D48" s="239"/>
-      <c r="E48" s="239"/>
-      <c r="F48" s="239"/>
-      <c r="G48" s="239"/>
-      <c r="H48" s="239"/>
-      <c r="I48" s="239"/>
-      <c r="J48" s="239"/>
-      <c r="K48" s="239"/>
-      <c r="L48" s="239"/>
-      <c r="M48" s="239"/>
-      <c r="N48" s="240"/>
+      <c r="B48" s="242"/>
+      <c r="C48" s="243"/>
+      <c r="D48" s="243"/>
+      <c r="E48" s="243"/>
+      <c r="F48" s="243"/>
+      <c r="G48" s="243"/>
+      <c r="H48" s="243"/>
+      <c r="I48" s="243"/>
+      <c r="J48" s="243"/>
+      <c r="K48" s="243"/>
+      <c r="L48" s="243"/>
+      <c r="M48" s="243"/>
+      <c r="N48" s="244"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B49" s="238"/>
-      <c r="C49" s="239"/>
-      <c r="D49" s="239"/>
-      <c r="E49" s="239"/>
-      <c r="F49" s="239"/>
-      <c r="G49" s="239"/>
-      <c r="H49" s="239"/>
-      <c r="I49" s="239"/>
-      <c r="J49" s="239"/>
-      <c r="K49" s="239"/>
-      <c r="L49" s="239"/>
-      <c r="M49" s="239"/>
-      <c r="N49" s="240"/>
+      <c r="B49" s="242"/>
+      <c r="C49" s="243"/>
+      <c r="D49" s="243"/>
+      <c r="E49" s="243"/>
+      <c r="F49" s="243"/>
+      <c r="G49" s="243"/>
+      <c r="H49" s="243"/>
+      <c r="I49" s="243"/>
+      <c r="J49" s="243"/>
+      <c r="K49" s="243"/>
+      <c r="L49" s="243"/>
+      <c r="M49" s="243"/>
+      <c r="N49" s="244"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B50" s="238"/>
-      <c r="C50" s="239"/>
-      <c r="D50" s="239"/>
-      <c r="E50" s="239"/>
-      <c r="F50" s="239"/>
-      <c r="G50" s="239"/>
-      <c r="H50" s="239"/>
-      <c r="I50" s="239"/>
-      <c r="J50" s="239"/>
-      <c r="K50" s="239"/>
-      <c r="L50" s="239"/>
-      <c r="M50" s="239"/>
-      <c r="N50" s="240"/>
+      <c r="B50" s="242"/>
+      <c r="C50" s="243"/>
+      <c r="D50" s="243"/>
+      <c r="E50" s="243"/>
+      <c r="F50" s="243"/>
+      <c r="G50" s="243"/>
+      <c r="H50" s="243"/>
+      <c r="I50" s="243"/>
+      <c r="J50" s="243"/>
+      <c r="K50" s="243"/>
+      <c r="L50" s="243"/>
+      <c r="M50" s="243"/>
+      <c r="N50" s="244"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B51" s="238"/>
-      <c r="C51" s="239"/>
-      <c r="D51" s="239"/>
-      <c r="E51" s="239"/>
-      <c r="F51" s="239"/>
-      <c r="G51" s="239"/>
-      <c r="H51" s="239"/>
-      <c r="I51" s="239"/>
-      <c r="J51" s="239"/>
-      <c r="K51" s="239"/>
-      <c r="L51" s="239"/>
-      <c r="M51" s="239"/>
-      <c r="N51" s="240"/>
+      <c r="B51" s="242"/>
+      <c r="C51" s="243"/>
+      <c r="D51" s="243"/>
+      <c r="E51" s="243"/>
+      <c r="F51" s="243"/>
+      <c r="G51" s="243"/>
+      <c r="H51" s="243"/>
+      <c r="I51" s="243"/>
+      <c r="J51" s="243"/>
+      <c r="K51" s="243"/>
+      <c r="L51" s="243"/>
+      <c r="M51" s="243"/>
+      <c r="N51" s="244"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="74"/>
-      <c r="B52" s="247" t="s">
+      <c r="B52" s="251" t="s">
         <v>82</v>
       </c>
-      <c r="C52" s="247"/>
-      <c r="D52" s="247"/>
-      <c r="E52" s="247"/>
-      <c r="F52" s="247"/>
-      <c r="G52" s="247"/>
-      <c r="H52" s="247"/>
-      <c r="I52" s="247"/>
-      <c r="J52" s="247"/>
-      <c r="K52" s="247"/>
-      <c r="L52" s="247"/>
-      <c r="M52" s="247"/>
-      <c r="N52" s="248"/>
+      <c r="C52" s="251"/>
+      <c r="D52" s="251"/>
+      <c r="E52" s="251"/>
+      <c r="F52" s="251"/>
+      <c r="G52" s="251"/>
+      <c r="H52" s="251"/>
+      <c r="I52" s="251"/>
+      <c r="J52" s="251"/>
+      <c r="K52" s="251"/>
+      <c r="L52" s="251"/>
+      <c r="M52" s="251"/>
+      <c r="N52" s="252"/>
     </row>
     <row r="53" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="74"/>
@@ -5926,19 +5926,19 @@
     </row>
     <row r="54" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="92"/>
-      <c r="C54" s="249" t="s">
+      <c r="C54" s="253" t="s">
         <v>83</v>
       </c>
-      <c r="D54" s="250"/>
-      <c r="E54" s="250"/>
-      <c r="F54" s="250"/>
-      <c r="G54" s="250"/>
-      <c r="I54" s="249" t="s">
+      <c r="D54" s="254"/>
+      <c r="E54" s="254"/>
+      <c r="F54" s="254"/>
+      <c r="G54" s="254"/>
+      <c r="I54" s="253" t="s">
         <v>84</v>
       </c>
-      <c r="J54" s="250"/>
-      <c r="K54" s="250"/>
-      <c r="L54" s="250"/>
+      <c r="J54" s="254"/>
+      <c r="K54" s="254"/>
+      <c r="L54" s="254"/>
       <c r="N54" s="74"/>
       <c r="O54" s="74"/>
     </row>
@@ -5952,15 +5952,15 @@
       <c r="C56" t="s">
         <v>85</v>
       </c>
-      <c r="E56" s="246"/>
-      <c r="F56" s="246"/>
-      <c r="G56" s="246"/>
+      <c r="E56" s="250"/>
+      <c r="F56" s="250"/>
+      <c r="G56" s="250"/>
       <c r="I56" t="s">
         <v>85</v>
       </c>
-      <c r="J56" s="246"/>
-      <c r="K56" s="246"/>
-      <c r="L56" s="246"/>
+      <c r="J56" s="250"/>
+      <c r="K56" s="250"/>
+      <c r="L56" s="250"/>
       <c r="N56" s="74"/>
       <c r="O56" s="74"/>
     </row>
@@ -5969,15 +5969,15 @@
       <c r="C57" t="s">
         <v>86</v>
       </c>
-      <c r="E57" s="246"/>
-      <c r="F57" s="246"/>
-      <c r="G57" s="246"/>
+      <c r="E57" s="250"/>
+      <c r="F57" s="250"/>
+      <c r="G57" s="250"/>
       <c r="I57" t="s">
         <v>86</v>
       </c>
-      <c r="J57" s="246"/>
-      <c r="K57" s="246"/>
-      <c r="L57" s="246"/>
+      <c r="J57" s="250"/>
+      <c r="K57" s="250"/>
+      <c r="L57" s="250"/>
       <c r="N57" s="74"/>
       <c r="O57" s="74"/>
     </row>
@@ -5986,15 +5986,15 @@
       <c r="C58" t="s">
         <v>87</v>
       </c>
-      <c r="E58" s="246"/>
-      <c r="F58" s="246"/>
-      <c r="G58" s="246"/>
+      <c r="E58" s="250"/>
+      <c r="F58" s="250"/>
+      <c r="G58" s="250"/>
       <c r="I58" t="s">
         <v>87</v>
       </c>
-      <c r="J58" s="246"/>
-      <c r="K58" s="246"/>
-      <c r="L58" s="246"/>
+      <c r="J58" s="250"/>
+      <c r="K58" s="250"/>
+      <c r="L58" s="250"/>
       <c r="N58" s="74"/>
       <c r="O58" s="74"/>
     </row>
@@ -6115,55 +6115,55 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E2" s="203" t="s">
+      <c r="E2" s="207" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="203"/>
-      <c r="G2" s="203"/>
-      <c r="H2" s="203"/>
-      <c r="I2" s="203"/>
-      <c r="J2" s="203"/>
+      <c r="F2" s="207"/>
+      <c r="G2" s="207"/>
+      <c r="H2" s="207"/>
+      <c r="I2" s="207"/>
+      <c r="J2" s="207"/>
       <c r="L2" s="112" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="3" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E3" s="204" t="s">
+      <c r="E3" s="208" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="204"/>
-      <c r="G3" s="204"/>
-      <c r="H3" s="204"/>
-      <c r="I3" s="204"/>
-      <c r="J3" s="204"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="208"/>
+      <c r="H3" s="208"/>
+      <c r="I3" s="208"/>
+      <c r="J3" s="208"/>
     </row>
     <row r="4" spans="2:14" ht="4.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:14" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="205" t="s">
+      <c r="B5" s="209" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="206"/>
-      <c r="D5" s="206"/>
-      <c r="E5" s="206"/>
-      <c r="F5" s="206"/>
-      <c r="G5" s="206"/>
-      <c r="H5" s="206"/>
-      <c r="I5" s="206"/>
-      <c r="J5" s="206"/>
-      <c r="K5" s="206"/>
-      <c r="L5" s="206"/>
-      <c r="M5" s="206"/>
-      <c r="N5" s="207"/>
+      <c r="C5" s="210"/>
+      <c r="D5" s="210"/>
+      <c r="E5" s="210"/>
+      <c r="F5" s="210"/>
+      <c r="G5" s="210"/>
+      <c r="H5" s="210"/>
+      <c r="I5" s="210"/>
+      <c r="J5" s="210"/>
+      <c r="K5" s="210"/>
+      <c r="L5" s="210"/>
+      <c r="M5" s="210"/>
+      <c r="N5" s="211"/>
     </row>
     <row r="6" spans="2:14" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="75"/>
       <c r="N6" s="74"/>
     </row>
     <row r="7" spans="2:14" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="208" t="s">
+      <c r="B7" s="212" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="209"/>
+      <c r="C7" s="213"/>
       <c r="D7" s="105"/>
       <c r="E7" s="107"/>
       <c r="F7" s="107"/>
@@ -6183,10 +6183,10 @@
       <c r="N8" s="74"/>
     </row>
     <row r="9" spans="2:14" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="208" t="s">
+      <c r="B9" s="212" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="209"/>
+      <c r="C9" s="213"/>
       <c r="D9" s="105"/>
       <c r="E9" s="107"/>
       <c r="F9" s="107"/>
@@ -6206,52 +6206,52 @@
       <c r="N10" s="74"/>
     </row>
     <row r="11" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="268" t="s">
+      <c r="B11" s="272" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="269"/>
+      <c r="C11" s="273"/>
       <c r="D11" s="106"/>
-      <c r="E11" s="257" t="s">
+      <c r="E11" s="261" t="s">
         <v>89</v>
       </c>
-      <c r="F11" s="258"/>
-      <c r="G11" s="258"/>
-      <c r="H11" s="258"/>
-      <c r="I11" s="258"/>
-      <c r="J11" s="258"/>
-      <c r="K11" s="258"/>
-      <c r="L11" s="258"/>
-      <c r="M11" s="259"/>
+      <c r="F11" s="262"/>
+      <c r="G11" s="262"/>
+      <c r="H11" s="262"/>
+      <c r="I11" s="262"/>
+      <c r="J11" s="262"/>
+      <c r="K11" s="262"/>
+      <c r="L11" s="262"/>
+      <c r="M11" s="263"/>
       <c r="N11" s="81"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="251"/>
-      <c r="C12" s="252"/>
+      <c r="B12" s="255"/>
+      <c r="C12" s="256"/>
       <c r="D12" s="106"/>
-      <c r="E12" s="251"/>
-      <c r="F12" s="255"/>
-      <c r="G12" s="255"/>
-      <c r="H12" s="255"/>
-      <c r="I12" s="255"/>
-      <c r="J12" s="255"/>
-      <c r="K12" s="255"/>
-      <c r="L12" s="255"/>
-      <c r="M12" s="252"/>
+      <c r="E12" s="255"/>
+      <c r="F12" s="259"/>
+      <c r="G12" s="259"/>
+      <c r="H12" s="259"/>
+      <c r="I12" s="259"/>
+      <c r="J12" s="259"/>
+      <c r="K12" s="259"/>
+      <c r="L12" s="259"/>
+      <c r="M12" s="256"/>
       <c r="N12" s="81"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="253"/>
-      <c r="C13" s="254"/>
+      <c r="B13" s="257"/>
+      <c r="C13" s="258"/>
       <c r="D13" s="106"/>
-      <c r="E13" s="253"/>
-      <c r="F13" s="256"/>
-      <c r="G13" s="256"/>
-      <c r="H13" s="256"/>
-      <c r="I13" s="256"/>
-      <c r="J13" s="256"/>
-      <c r="K13" s="256"/>
-      <c r="L13" s="256"/>
-      <c r="M13" s="254"/>
+      <c r="E13" s="257"/>
+      <c r="F13" s="260"/>
+      <c r="G13" s="260"/>
+      <c r="H13" s="260"/>
+      <c r="I13" s="260"/>
+      <c r="J13" s="260"/>
+      <c r="K13" s="260"/>
+      <c r="L13" s="260"/>
+      <c r="M13" s="258"/>
       <c r="N13" s="81"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
@@ -6260,45 +6260,45 @@
       <c r="N14" s="74"/>
     </row>
     <row r="15" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="208" t="s">
+      <c r="B15" s="212" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="209"/>
+      <c r="C15" s="213"/>
       <c r="D15" s="105"/>
-      <c r="E15" s="260"/>
-      <c r="F15" s="261"/>
-      <c r="G15" s="262"/>
+      <c r="E15" s="264"/>
+      <c r="F15" s="265"/>
+      <c r="G15" s="266"/>
       <c r="H15" s="78"/>
-      <c r="I15" s="209" t="s">
+      <c r="I15" s="213" t="s">
         <v>66</v>
       </c>
-      <c r="J15" s="209"/>
-      <c r="K15" s="228"/>
-      <c r="L15" s="263"/>
-      <c r="M15" s="264"/>
+      <c r="J15" s="213"/>
+      <c r="K15" s="232"/>
+      <c r="L15" s="267"/>
+      <c r="M15" s="268"/>
       <c r="N15" s="82"/>
     </row>
     <row r="16" spans="2:14" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="75"/>
       <c r="N16" s="74"/>
     </row>
-    <row r="17" spans="2:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="208" t="s">
+    <row r="17" spans="2:14" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="212" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="209"/>
+      <c r="C17" s="213"/>
       <c r="D17" s="105"/>
-      <c r="E17" s="265"/>
-      <c r="F17" s="266"/>
-      <c r="G17" s="267"/>
+      <c r="E17" s="269"/>
+      <c r="F17" s="270"/>
+      <c r="G17" s="271"/>
       <c r="H17" s="79"/>
-      <c r="I17" s="209" t="s">
+      <c r="I17" s="213" t="s">
         <v>68</v>
       </c>
-      <c r="J17" s="209"/>
-      <c r="K17" s="231"/>
-      <c r="L17" s="229"/>
-      <c r="M17" s="230"/>
+      <c r="J17" s="213"/>
+      <c r="K17" s="235"/>
+      <c r="L17" s="233"/>
+      <c r="M17" s="234"/>
       <c r="N17" s="82"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.3">
@@ -6317,153 +6317,153 @@
       <c r="N20" s="74"/>
     </row>
     <row r="21" spans="2:14" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="205" t="s">
+      <c r="B21" s="209" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="206"/>
-      <c r="D21" s="206"/>
-      <c r="E21" s="206"/>
-      <c r="F21" s="206"/>
-      <c r="G21" s="206"/>
-      <c r="H21" s="206"/>
-      <c r="I21" s="206"/>
-      <c r="J21" s="206"/>
-      <c r="K21" s="206"/>
-      <c r="L21" s="206"/>
-      <c r="M21" s="206"/>
-      <c r="N21" s="207"/>
+      <c r="C21" s="210"/>
+      <c r="D21" s="210"/>
+      <c r="E21" s="210"/>
+      <c r="F21" s="210"/>
+      <c r="G21" s="210"/>
+      <c r="H21" s="210"/>
+      <c r="I21" s="210"/>
+      <c r="J21" s="210"/>
+      <c r="K21" s="210"/>
+      <c r="L21" s="210"/>
+      <c r="M21" s="210"/>
+      <c r="N21" s="211"/>
     </row>
     <row r="22" spans="2:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="212" t="s">
+      <c r="B22" s="216" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="213"/>
-      <c r="D22" s="213"/>
-      <c r="E22" s="213"/>
-      <c r="F22" s="213"/>
-      <c r="G22" s="213"/>
-      <c r="H22" s="213"/>
-      <c r="I22" s="213"/>
-      <c r="J22" s="213"/>
-      <c r="K22" s="213"/>
-      <c r="L22" s="213"/>
-      <c r="M22" s="213"/>
-      <c r="N22" s="214"/>
+      <c r="C22" s="217"/>
+      <c r="D22" s="217"/>
+      <c r="E22" s="217"/>
+      <c r="F22" s="217"/>
+      <c r="G22" s="217"/>
+      <c r="H22" s="217"/>
+      <c r="I22" s="217"/>
+      <c r="J22" s="217"/>
+      <c r="K22" s="217"/>
+      <c r="L22" s="217"/>
+      <c r="M22" s="217"/>
+      <c r="N22" s="218"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B23" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="235" t="s">
+      <c r="C23" s="239" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="236"/>
-      <c r="E23" s="236"/>
-      <c r="F23" s="236"/>
-      <c r="G23" s="236"/>
-      <c r="H23" s="237"/>
-      <c r="I23" s="235" t="s">
+      <c r="D23" s="240"/>
+      <c r="E23" s="240"/>
+      <c r="F23" s="240"/>
+      <c r="G23" s="240"/>
+      <c r="H23" s="241"/>
+      <c r="I23" s="239" t="s">
         <v>73</v>
       </c>
-      <c r="J23" s="237"/>
-      <c r="K23" s="235" t="s">
+      <c r="J23" s="241"/>
+      <c r="K23" s="239" t="s">
         <v>74</v>
       </c>
-      <c r="L23" s="236"/>
-      <c r="M23" s="236"/>
-      <c r="N23" s="237"/>
+      <c r="L23" s="240"/>
+      <c r="M23" s="240"/>
+      <c r="N23" s="241"/>
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B24" s="73">
         <v>1</v>
       </c>
-      <c r="C24" s="232" t="s">
+      <c r="C24" s="236" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="233"/>
-      <c r="E24" s="233"/>
-      <c r="F24" s="233"/>
-      <c r="G24" s="233"/>
-      <c r="H24" s="234"/>
-      <c r="I24" s="232"/>
-      <c r="J24" s="234"/>
-      <c r="K24" s="232"/>
-      <c r="L24" s="233"/>
-      <c r="M24" s="233"/>
+      <c r="D24" s="237"/>
+      <c r="E24" s="237"/>
+      <c r="F24" s="237"/>
+      <c r="G24" s="237"/>
+      <c r="H24" s="238"/>
+      <c r="I24" s="236"/>
+      <c r="J24" s="238"/>
+      <c r="K24" s="236"/>
+      <c r="L24" s="237"/>
+      <c r="M24" s="237"/>
       <c r="N24" s="85"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B25" s="73">
         <v>2</v>
       </c>
-      <c r="C25" s="232" t="s">
+      <c r="C25" s="236" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="233"/>
-      <c r="E25" s="233"/>
-      <c r="F25" s="233"/>
-      <c r="G25" s="233"/>
-      <c r="H25" s="234"/>
-      <c r="I25" s="232"/>
-      <c r="J25" s="234"/>
-      <c r="K25" s="232"/>
-      <c r="L25" s="233"/>
-      <c r="M25" s="233"/>
+      <c r="D25" s="237"/>
+      <c r="E25" s="237"/>
+      <c r="F25" s="237"/>
+      <c r="G25" s="237"/>
+      <c r="H25" s="238"/>
+      <c r="I25" s="236"/>
+      <c r="J25" s="238"/>
+      <c r="K25" s="236"/>
+      <c r="L25" s="237"/>
+      <c r="M25" s="237"/>
       <c r="N25" s="86"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B26" s="73">
         <v>3</v>
       </c>
-      <c r="C26" s="232" t="s">
+      <c r="C26" s="236" t="s">
         <v>77</v>
       </c>
-      <c r="D26" s="233"/>
-      <c r="E26" s="233"/>
-      <c r="F26" s="233"/>
-      <c r="G26" s="233"/>
-      <c r="H26" s="234"/>
-      <c r="K26" s="232"/>
-      <c r="L26" s="233"/>
-      <c r="M26" s="233"/>
+      <c r="D26" s="237"/>
+      <c r="E26" s="237"/>
+      <c r="F26" s="237"/>
+      <c r="G26" s="237"/>
+      <c r="H26" s="238"/>
+      <c r="K26" s="236"/>
+      <c r="L26" s="237"/>
+      <c r="M26" s="237"/>
       <c r="N26" s="86"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B27" s="73">
         <v>4</v>
       </c>
-      <c r="C27" s="232" t="s">
+      <c r="C27" s="236" t="s">
         <v>78</v>
       </c>
-      <c r="D27" s="233"/>
-      <c r="E27" s="233"/>
-      <c r="F27" s="233"/>
-      <c r="G27" s="233"/>
-      <c r="H27" s="234"/>
-      <c r="I27" s="232"/>
-      <c r="J27" s="234"/>
-      <c r="K27" s="232"/>
-      <c r="L27" s="233"/>
-      <c r="M27" s="233"/>
+      <c r="D27" s="237"/>
+      <c r="E27" s="237"/>
+      <c r="F27" s="237"/>
+      <c r="G27" s="237"/>
+      <c r="H27" s="238"/>
+      <c r="I27" s="236"/>
+      <c r="J27" s="238"/>
+      <c r="K27" s="236"/>
+      <c r="L27" s="237"/>
+      <c r="M27" s="237"/>
       <c r="N27" s="86"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B28" s="73">
         <v>5</v>
       </c>
-      <c r="C28" s="232" t="s">
+      <c r="C28" s="236" t="s">
         <v>79</v>
       </c>
-      <c r="D28" s="233"/>
-      <c r="E28" s="233"/>
-      <c r="F28" s="233"/>
-      <c r="G28" s="233"/>
-      <c r="H28" s="234"/>
-      <c r="I28" s="232"/>
-      <c r="J28" s="234"/>
-      <c r="K28" s="232"/>
-      <c r="L28" s="233"/>
-      <c r="M28" s="233"/>
+      <c r="D28" s="237"/>
+      <c r="E28" s="237"/>
+      <c r="F28" s="237"/>
+      <c r="G28" s="237"/>
+      <c r="H28" s="238"/>
+      <c r="I28" s="236"/>
+      <c r="J28" s="238"/>
+      <c r="K28" s="236"/>
+      <c r="L28" s="237"/>
+      <c r="M28" s="237"/>
       <c r="N28" s="86"/>
     </row>
     <row r="29" spans="2:14" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6471,200 +6471,200 @@
       <c r="N29" s="74"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B30" s="241" t="s">
+      <c r="B30" s="245" t="s">
         <v>80</v>
       </c>
-      <c r="C30" s="242"/>
-      <c r="D30" s="242"/>
-      <c r="E30" s="242"/>
-      <c r="F30" s="242"/>
-      <c r="G30" s="242"/>
-      <c r="H30" s="242"/>
-      <c r="I30" s="242"/>
-      <c r="J30" s="242"/>
-      <c r="K30" s="242"/>
-      <c r="L30" s="242"/>
-      <c r="M30" s="242"/>
-      <c r="N30" s="243"/>
+      <c r="C30" s="246"/>
+      <c r="D30" s="246"/>
+      <c r="E30" s="246"/>
+      <c r="F30" s="246"/>
+      <c r="G30" s="246"/>
+      <c r="H30" s="246"/>
+      <c r="I30" s="246"/>
+      <c r="J30" s="246"/>
+      <c r="K30" s="246"/>
+      <c r="L30" s="246"/>
+      <c r="M30" s="246"/>
+      <c r="N30" s="247"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B31" s="272"/>
-      <c r="C31" s="273"/>
-      <c r="D31" s="273"/>
-      <c r="E31" s="273"/>
-      <c r="F31" s="273"/>
-      <c r="G31" s="273"/>
-      <c r="H31" s="273"/>
-      <c r="I31" s="273"/>
-      <c r="J31" s="273"/>
-      <c r="K31" s="273"/>
-      <c r="L31" s="273"/>
-      <c r="M31" s="273"/>
+      <c r="B31" s="115"/>
+      <c r="C31" s="116"/>
+      <c r="D31" s="116"/>
+      <c r="E31" s="116"/>
+      <c r="F31" s="116"/>
+      <c r="G31" s="116"/>
+      <c r="H31" s="116"/>
+      <c r="I31" s="116"/>
+      <c r="J31" s="116"/>
+      <c r="K31" s="116"/>
+      <c r="L31" s="116"/>
+      <c r="M31" s="116"/>
       <c r="N31" s="84"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B32" s="270"/>
-      <c r="C32" s="271"/>
-      <c r="D32" s="271"/>
-      <c r="E32" s="271"/>
-      <c r="F32" s="271"/>
-      <c r="G32" s="271"/>
-      <c r="H32" s="271"/>
-      <c r="I32" s="271"/>
-      <c r="J32" s="271"/>
-      <c r="K32" s="271"/>
-      <c r="L32" s="271"/>
-      <c r="M32" s="271"/>
+      <c r="B32" s="113"/>
+      <c r="C32" s="114"/>
+      <c r="D32" s="114"/>
+      <c r="E32" s="114"/>
+      <c r="F32" s="114"/>
+      <c r="G32" s="114"/>
+      <c r="H32" s="114"/>
+      <c r="I32" s="114"/>
+      <c r="J32" s="114"/>
+      <c r="K32" s="114"/>
+      <c r="L32" s="114"/>
+      <c r="M32" s="114"/>
       <c r="N32" s="82"/>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B33" s="270"/>
-      <c r="C33" s="271"/>
-      <c r="D33" s="271"/>
-      <c r="E33" s="271"/>
-      <c r="F33" s="271"/>
-      <c r="G33" s="271"/>
-      <c r="H33" s="271"/>
-      <c r="I33" s="271"/>
-      <c r="J33" s="271"/>
-      <c r="K33" s="271"/>
-      <c r="L33" s="271"/>
-      <c r="M33" s="271"/>
+      <c r="B33" s="113"/>
+      <c r="C33" s="114"/>
+      <c r="D33" s="114"/>
+      <c r="E33" s="114"/>
+      <c r="F33" s="114"/>
+      <c r="G33" s="114"/>
+      <c r="H33" s="114"/>
+      <c r="I33" s="114"/>
+      <c r="J33" s="114"/>
+      <c r="K33" s="114"/>
+      <c r="L33" s="114"/>
+      <c r="M33" s="114"/>
       <c r="N33" s="82"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B34" s="270"/>
-      <c r="C34" s="271"/>
-      <c r="D34" s="271"/>
-      <c r="E34" s="271"/>
-      <c r="F34" s="271"/>
-      <c r="G34" s="271"/>
-      <c r="H34" s="271"/>
-      <c r="I34" s="271"/>
-      <c r="J34" s="271"/>
-      <c r="K34" s="271"/>
-      <c r="L34" s="271"/>
-      <c r="M34" s="271"/>
+      <c r="B34" s="113"/>
+      <c r="C34" s="114"/>
+      <c r="D34" s="114"/>
+      <c r="E34" s="114"/>
+      <c r="F34" s="114"/>
+      <c r="G34" s="114"/>
+      <c r="H34" s="114"/>
+      <c r="I34" s="114"/>
+      <c r="J34" s="114"/>
+      <c r="K34" s="114"/>
+      <c r="L34" s="114"/>
+      <c r="M34" s="114"/>
       <c r="N34" s="82"/>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B35" s="270"/>
-      <c r="C35" s="271"/>
-      <c r="D35" s="271"/>
-      <c r="E35" s="271"/>
-      <c r="F35" s="271"/>
-      <c r="G35" s="271"/>
-      <c r="H35" s="271"/>
-      <c r="I35" s="271"/>
-      <c r="J35" s="271"/>
-      <c r="K35" s="271"/>
-      <c r="L35" s="271"/>
-      <c r="M35" s="271"/>
+      <c r="B35" s="113"/>
+      <c r="C35" s="114"/>
+      <c r="D35" s="114"/>
+      <c r="E35" s="114"/>
+      <c r="F35" s="114"/>
+      <c r="G35" s="114"/>
+      <c r="H35" s="114"/>
+      <c r="I35" s="114"/>
+      <c r="J35" s="114"/>
+      <c r="K35" s="114"/>
+      <c r="L35" s="114"/>
+      <c r="M35" s="114"/>
       <c r="N35" s="82"/>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B36" s="270"/>
-      <c r="C36" s="271"/>
-      <c r="D36" s="271"/>
-      <c r="E36" s="271"/>
-      <c r="F36" s="271"/>
-      <c r="G36" s="271"/>
-      <c r="H36" s="271"/>
-      <c r="I36" s="271"/>
-      <c r="J36" s="271"/>
-      <c r="K36" s="271"/>
-      <c r="L36" s="271"/>
-      <c r="M36" s="271"/>
+      <c r="B36" s="113"/>
+      <c r="C36" s="114"/>
+      <c r="D36" s="114"/>
+      <c r="E36" s="114"/>
+      <c r="F36" s="114"/>
+      <c r="G36" s="114"/>
+      <c r="H36" s="114"/>
+      <c r="I36" s="114"/>
+      <c r="J36" s="114"/>
+      <c r="K36" s="114"/>
+      <c r="L36" s="114"/>
+      <c r="M36" s="114"/>
       <c r="N36" s="82"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B37" s="270"/>
-      <c r="C37" s="271"/>
-      <c r="D37" s="271"/>
-      <c r="E37" s="271"/>
-      <c r="F37" s="271"/>
-      <c r="G37" s="271"/>
-      <c r="H37" s="271"/>
-      <c r="I37" s="271"/>
-      <c r="J37" s="271"/>
-      <c r="K37" s="271"/>
-      <c r="L37" s="271"/>
-      <c r="M37" s="271"/>
+      <c r="B37" s="113"/>
+      <c r="C37" s="114"/>
+      <c r="D37" s="114"/>
+      <c r="E37" s="114"/>
+      <c r="F37" s="114"/>
+      <c r="G37" s="114"/>
+      <c r="H37" s="114"/>
+      <c r="I37" s="114"/>
+      <c r="J37" s="114"/>
+      <c r="K37" s="114"/>
+      <c r="L37" s="114"/>
+      <c r="M37" s="114"/>
       <c r="N37" s="82"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B38" s="270"/>
-      <c r="C38" s="271"/>
-      <c r="D38" s="271"/>
-      <c r="E38" s="271"/>
-      <c r="F38" s="271"/>
-      <c r="G38" s="271"/>
-      <c r="H38" s="271"/>
-      <c r="I38" s="271"/>
-      <c r="J38" s="271"/>
-      <c r="K38" s="271"/>
-      <c r="L38" s="271"/>
-      <c r="M38" s="271"/>
+      <c r="B38" s="113"/>
+      <c r="C38" s="114"/>
+      <c r="D38" s="114"/>
+      <c r="E38" s="114"/>
+      <c r="F38" s="114"/>
+      <c r="G38" s="114"/>
+      <c r="H38" s="114"/>
+      <c r="I38" s="114"/>
+      <c r="J38" s="114"/>
+      <c r="K38" s="114"/>
+      <c r="L38" s="114"/>
+      <c r="M38" s="114"/>
       <c r="N38" s="82"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B39" s="270"/>
-      <c r="C39" s="271"/>
-      <c r="D39" s="271"/>
-      <c r="E39" s="271"/>
-      <c r="F39" s="271"/>
-      <c r="G39" s="271"/>
-      <c r="H39" s="271"/>
-      <c r="I39" s="271"/>
-      <c r="J39" s="271"/>
-      <c r="K39" s="271"/>
-      <c r="L39" s="271"/>
-      <c r="M39" s="271"/>
+      <c r="B39" s="113"/>
+      <c r="C39" s="114"/>
+      <c r="D39" s="114"/>
+      <c r="E39" s="114"/>
+      <c r="F39" s="114"/>
+      <c r="G39" s="114"/>
+      <c r="H39" s="114"/>
+      <c r="I39" s="114"/>
+      <c r="J39" s="114"/>
+      <c r="K39" s="114"/>
+      <c r="L39" s="114"/>
+      <c r="M39" s="114"/>
       <c r="N39" s="82"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B40" s="270"/>
-      <c r="C40" s="271"/>
-      <c r="D40" s="271"/>
-      <c r="E40" s="271"/>
-      <c r="F40" s="271"/>
-      <c r="G40" s="271"/>
-      <c r="H40" s="271"/>
-      <c r="I40" s="271"/>
-      <c r="J40" s="271"/>
-      <c r="K40" s="271"/>
-      <c r="L40" s="271"/>
-      <c r="M40" s="271"/>
+      <c r="B40" s="113"/>
+      <c r="C40" s="114"/>
+      <c r="D40" s="114"/>
+      <c r="E40" s="114"/>
+      <c r="F40" s="114"/>
+      <c r="G40" s="114"/>
+      <c r="H40" s="114"/>
+      <c r="I40" s="114"/>
+      <c r="J40" s="114"/>
+      <c r="K40" s="114"/>
+      <c r="L40" s="114"/>
+      <c r="M40" s="114"/>
       <c r="N40" s="82"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B41" s="270"/>
-      <c r="C41" s="271"/>
-      <c r="D41" s="271"/>
-      <c r="E41" s="271"/>
-      <c r="F41" s="271"/>
-      <c r="G41" s="271"/>
-      <c r="H41" s="271"/>
-      <c r="I41" s="271"/>
-      <c r="J41" s="271"/>
-      <c r="K41" s="271"/>
-      <c r="L41" s="271"/>
-      <c r="M41" s="271"/>
+      <c r="B41" s="113"/>
+      <c r="C41" s="114"/>
+      <c r="D41" s="114"/>
+      <c r="E41" s="114"/>
+      <c r="F41" s="114"/>
+      <c r="G41" s="114"/>
+      <c r="H41" s="114"/>
+      <c r="I41" s="114"/>
+      <c r="J41" s="114"/>
+      <c r="K41" s="114"/>
+      <c r="L41" s="114"/>
+      <c r="M41" s="114"/>
       <c r="N41" s="82"/>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B42" s="270"/>
-      <c r="C42" s="271"/>
-      <c r="D42" s="271"/>
-      <c r="E42" s="271"/>
-      <c r="F42" s="271"/>
-      <c r="G42" s="271"/>
-      <c r="H42" s="271"/>
-      <c r="I42" s="271"/>
-      <c r="J42" s="271"/>
-      <c r="K42" s="271"/>
-      <c r="L42" s="271"/>
-      <c r="M42" s="271"/>
+      <c r="B42" s="113"/>
+      <c r="C42" s="114"/>
+      <c r="D42" s="114"/>
+      <c r="E42" s="114"/>
+      <c r="F42" s="114"/>
+      <c r="G42" s="114"/>
+      <c r="H42" s="114"/>
+      <c r="I42" s="114"/>
+      <c r="J42" s="114"/>
+      <c r="K42" s="114"/>
+      <c r="L42" s="114"/>
+      <c r="M42" s="114"/>
       <c r="N42" s="82"/>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.3">
@@ -6687,131 +6687,131 @@
       <c r="N44" s="74"/>
     </row>
     <row r="45" spans="2:14" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B45" s="205" t="s">
+      <c r="B45" s="209" t="s">
         <v>81</v>
       </c>
-      <c r="C45" s="206"/>
-      <c r="D45" s="206"/>
-      <c r="E45" s="206"/>
-      <c r="F45" s="206"/>
-      <c r="G45" s="206"/>
-      <c r="H45" s="206"/>
-      <c r="I45" s="206"/>
-      <c r="J45" s="206"/>
-      <c r="K45" s="206"/>
-      <c r="L45" s="206"/>
-      <c r="M45" s="206"/>
-      <c r="N45" s="207"/>
+      <c r="C45" s="210"/>
+      <c r="D45" s="210"/>
+      <c r="E45" s="210"/>
+      <c r="F45" s="210"/>
+      <c r="G45" s="210"/>
+      <c r="H45" s="210"/>
+      <c r="I45" s="210"/>
+      <c r="J45" s="210"/>
+      <c r="K45" s="210"/>
+      <c r="L45" s="210"/>
+      <c r="M45" s="210"/>
+      <c r="N45" s="211"/>
     </row>
     <row r="46" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="238" t="s">
+      <c r="B46" s="242" t="s">
         <v>34</v>
       </c>
-      <c r="C46" s="239"/>
-      <c r="D46" s="239"/>
-      <c r="E46" s="239"/>
-      <c r="F46" s="239"/>
-      <c r="G46" s="239"/>
-      <c r="H46" s="239"/>
-      <c r="I46" s="239"/>
-      <c r="J46" s="239"/>
-      <c r="K46" s="239"/>
-      <c r="L46" s="239"/>
-      <c r="M46" s="239"/>
-      <c r="N46" s="240"/>
+      <c r="C46" s="243"/>
+      <c r="D46" s="243"/>
+      <c r="E46" s="243"/>
+      <c r="F46" s="243"/>
+      <c r="G46" s="243"/>
+      <c r="H46" s="243"/>
+      <c r="I46" s="243"/>
+      <c r="J46" s="243"/>
+      <c r="K46" s="243"/>
+      <c r="L46" s="243"/>
+      <c r="M46" s="243"/>
+      <c r="N46" s="244"/>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B47" s="238"/>
-      <c r="C47" s="239"/>
-      <c r="D47" s="239"/>
-      <c r="E47" s="239"/>
-      <c r="F47" s="239"/>
-      <c r="G47" s="239"/>
-      <c r="H47" s="239"/>
-      <c r="I47" s="239"/>
-      <c r="J47" s="239"/>
-      <c r="K47" s="239"/>
-      <c r="L47" s="239"/>
-      <c r="M47" s="239"/>
-      <c r="N47" s="240"/>
+      <c r="B47" s="242"/>
+      <c r="C47" s="243"/>
+      <c r="D47" s="243"/>
+      <c r="E47" s="243"/>
+      <c r="F47" s="243"/>
+      <c r="G47" s="243"/>
+      <c r="H47" s="243"/>
+      <c r="I47" s="243"/>
+      <c r="J47" s="243"/>
+      <c r="K47" s="243"/>
+      <c r="L47" s="243"/>
+      <c r="M47" s="243"/>
+      <c r="N47" s="244"/>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B48" s="238"/>
-      <c r="C48" s="239"/>
-      <c r="D48" s="239"/>
-      <c r="E48" s="239"/>
-      <c r="F48" s="239"/>
-      <c r="G48" s="239"/>
-      <c r="H48" s="239"/>
-      <c r="I48" s="239"/>
-      <c r="J48" s="239"/>
-      <c r="K48" s="239"/>
-      <c r="L48" s="239"/>
-      <c r="M48" s="239"/>
-      <c r="N48" s="240"/>
+      <c r="B48" s="242"/>
+      <c r="C48" s="243"/>
+      <c r="D48" s="243"/>
+      <c r="E48" s="243"/>
+      <c r="F48" s="243"/>
+      <c r="G48" s="243"/>
+      <c r="H48" s="243"/>
+      <c r="I48" s="243"/>
+      <c r="J48" s="243"/>
+      <c r="K48" s="243"/>
+      <c r="L48" s="243"/>
+      <c r="M48" s="243"/>
+      <c r="N48" s="244"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B49" s="238"/>
-      <c r="C49" s="239"/>
-      <c r="D49" s="239"/>
-      <c r="E49" s="239"/>
-      <c r="F49" s="239"/>
-      <c r="G49" s="239"/>
-      <c r="H49" s="239"/>
-      <c r="I49" s="239"/>
-      <c r="J49" s="239"/>
-      <c r="K49" s="239"/>
-      <c r="L49" s="239"/>
-      <c r="M49" s="239"/>
-      <c r="N49" s="240"/>
+      <c r="B49" s="242"/>
+      <c r="C49" s="243"/>
+      <c r="D49" s="243"/>
+      <c r="E49" s="243"/>
+      <c r="F49" s="243"/>
+      <c r="G49" s="243"/>
+      <c r="H49" s="243"/>
+      <c r="I49" s="243"/>
+      <c r="J49" s="243"/>
+      <c r="K49" s="243"/>
+      <c r="L49" s="243"/>
+      <c r="M49" s="243"/>
+      <c r="N49" s="244"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B50" s="238"/>
-      <c r="C50" s="239"/>
-      <c r="D50" s="239"/>
-      <c r="E50" s="239"/>
-      <c r="F50" s="239"/>
-      <c r="G50" s="239"/>
-      <c r="H50" s="239"/>
-      <c r="I50" s="239"/>
-      <c r="J50" s="239"/>
-      <c r="K50" s="239"/>
-      <c r="L50" s="239"/>
-      <c r="M50" s="239"/>
-      <c r="N50" s="240"/>
+      <c r="B50" s="242"/>
+      <c r="C50" s="243"/>
+      <c r="D50" s="243"/>
+      <c r="E50" s="243"/>
+      <c r="F50" s="243"/>
+      <c r="G50" s="243"/>
+      <c r="H50" s="243"/>
+      <c r="I50" s="243"/>
+      <c r="J50" s="243"/>
+      <c r="K50" s="243"/>
+      <c r="L50" s="243"/>
+      <c r="M50" s="243"/>
+      <c r="N50" s="244"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B51" s="238"/>
-      <c r="C51" s="239"/>
-      <c r="D51" s="239"/>
-      <c r="E51" s="239"/>
-      <c r="F51" s="239"/>
-      <c r="G51" s="239"/>
-      <c r="H51" s="239"/>
-      <c r="I51" s="239"/>
-      <c r="J51" s="239"/>
-      <c r="K51" s="239"/>
-      <c r="L51" s="239"/>
-      <c r="M51" s="239"/>
-      <c r="N51" s="240"/>
+      <c r="B51" s="242"/>
+      <c r="C51" s="243"/>
+      <c r="D51" s="243"/>
+      <c r="E51" s="243"/>
+      <c r="F51" s="243"/>
+      <c r="G51" s="243"/>
+      <c r="H51" s="243"/>
+      <c r="I51" s="243"/>
+      <c r="J51" s="243"/>
+      <c r="K51" s="243"/>
+      <c r="L51" s="243"/>
+      <c r="M51" s="243"/>
+      <c r="N51" s="244"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="74"/>
-      <c r="B52" s="247" t="s">
+      <c r="B52" s="251" t="s">
         <v>82</v>
       </c>
-      <c r="C52" s="247"/>
-      <c r="D52" s="247"/>
-      <c r="E52" s="247"/>
-      <c r="F52" s="247"/>
-      <c r="G52" s="247"/>
-      <c r="H52" s="247"/>
-      <c r="I52" s="247"/>
-      <c r="J52" s="247"/>
-      <c r="K52" s="247"/>
-      <c r="L52" s="247"/>
-      <c r="M52" s="247"/>
-      <c r="N52" s="248"/>
+      <c r="C52" s="251"/>
+      <c r="D52" s="251"/>
+      <c r="E52" s="251"/>
+      <c r="F52" s="251"/>
+      <c r="G52" s="251"/>
+      <c r="H52" s="251"/>
+      <c r="I52" s="251"/>
+      <c r="J52" s="251"/>
+      <c r="K52" s="251"/>
+      <c r="L52" s="251"/>
+      <c r="M52" s="251"/>
+      <c r="N52" s="252"/>
     </row>
     <row r="53" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="74"/>
@@ -6831,19 +6831,19 @@
     </row>
     <row r="54" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="92"/>
-      <c r="C54" s="249" t="s">
+      <c r="C54" s="253" t="s">
         <v>83</v>
       </c>
-      <c r="D54" s="250"/>
-      <c r="E54" s="250"/>
-      <c r="F54" s="250"/>
-      <c r="G54" s="250"/>
-      <c r="I54" s="249" t="s">
+      <c r="D54" s="254"/>
+      <c r="E54" s="254"/>
+      <c r="F54" s="254"/>
+      <c r="G54" s="254"/>
+      <c r="I54" s="253" t="s">
         <v>84</v>
       </c>
-      <c r="J54" s="250"/>
-      <c r="K54" s="250"/>
-      <c r="L54" s="250"/>
+      <c r="J54" s="254"/>
+      <c r="K54" s="254"/>
+      <c r="L54" s="254"/>
       <c r="N54" s="74"/>
       <c r="O54" s="74"/>
     </row>
@@ -6852,20 +6852,20 @@
       <c r="N55" s="74"/>
       <c r="O55" s="74"/>
     </row>
-    <row r="56" spans="1:15" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:15" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="92"/>
       <c r="C56" t="s">
         <v>85</v>
       </c>
-      <c r="E56" s="246"/>
-      <c r="F56" s="246"/>
-      <c r="G56" s="246"/>
+      <c r="E56" s="250"/>
+      <c r="F56" s="250"/>
+      <c r="G56" s="250"/>
       <c r="I56" t="s">
         <v>85</v>
       </c>
-      <c r="J56" s="246"/>
-      <c r="K56" s="246"/>
-      <c r="L56" s="246"/>
+      <c r="J56" s="250"/>
+      <c r="K56" s="250"/>
+      <c r="L56" s="250"/>
       <c r="N56" s="74"/>
       <c r="O56" s="74"/>
     </row>
@@ -6874,15 +6874,15 @@
       <c r="C57" t="s">
         <v>86</v>
       </c>
-      <c r="E57" s="246"/>
-      <c r="F57" s="246"/>
-      <c r="G57" s="246"/>
+      <c r="E57" s="250"/>
+      <c r="F57" s="250"/>
+      <c r="G57" s="250"/>
       <c r="I57" t="s">
         <v>86</v>
       </c>
-      <c r="J57" s="246"/>
-      <c r="K57" s="246"/>
-      <c r="L57" s="246"/>
+      <c r="J57" s="250"/>
+      <c r="K57" s="250"/>
+      <c r="L57" s="250"/>
       <c r="N57" s="74"/>
       <c r="O57" s="74"/>
     </row>
@@ -6891,15 +6891,15 @@
       <c r="C58" t="s">
         <v>87</v>
       </c>
-      <c r="E58" s="246"/>
-      <c r="F58" s="246"/>
-      <c r="G58" s="246"/>
+      <c r="E58" s="250"/>
+      <c r="F58" s="250"/>
+      <c r="G58" s="250"/>
       <c r="I58" t="s">
         <v>87</v>
       </c>
-      <c r="J58" s="246"/>
-      <c r="K58" s="246"/>
-      <c r="L58" s="246"/>
+      <c r="J58" s="250"/>
+      <c r="K58" s="250"/>
+      <c r="L58" s="250"/>
       <c r="N58" s="74"/>
       <c r="O58" s="74"/>
     </row>
@@ -6959,6 +6959,8 @@
     <mergeCell ref="C25:H25"/>
     <mergeCell ref="I25:J25"/>
     <mergeCell ref="K25:M25"/>
+    <mergeCell ref="B45:N45"/>
+    <mergeCell ref="C27:H27"/>
     <mergeCell ref="C26:H26"/>
     <mergeCell ref="K26:M26"/>
     <mergeCell ref="C23:H23"/>
@@ -6967,6 +6969,8 @@
     <mergeCell ref="C24:H24"/>
     <mergeCell ref="I24:J24"/>
     <mergeCell ref="K24:M24"/>
+    <mergeCell ref="K27:M27"/>
+    <mergeCell ref="B30:N30"/>
     <mergeCell ref="I27:J27"/>
     <mergeCell ref="E58:G58"/>
     <mergeCell ref="J58:L58"/>
@@ -6981,10 +6985,6 @@
     <mergeCell ref="C28:H28"/>
     <mergeCell ref="I28:J28"/>
     <mergeCell ref="K28:M28"/>
-    <mergeCell ref="B45:N45"/>
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="K27:M27"/>
-    <mergeCell ref="B30:N30"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.12" top="0.31496062992125984" bottom="0.31496062992125984" header="0" footer="0"/>
   <pageSetup scale="75" orientation="portrait" r:id="rId1"/>

</xml_diff>